<commit_message>
Publish credentials and harden Sheets fallback
</commit_message>
<xml_diff>
--- a/docs/Portfolio_Website_Content_Model.xlsx
+++ b/docs/Portfolio_Website_Content_Model.xlsx
@@ -25,13 +25,13 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'README'!$A$1:$B$7</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Site_Config'!$A$1:$E$7</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Site_Config'!$A$1:$E$8</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Home_Sections'!$A$1:$G$3</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Experience_Education'!$A$1:$L$5</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'DB_People'!$A$1:$H$109</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'DB_Publications'!$A$1:$X$44</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'DB_PublicationAuthor'!$A$1:$F$491</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'WEB_Publications'!$A$1:$X$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'WEB_Publications'!$A$1:$X$44</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'WEB_People'!$A$1:$D$109</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'Projects'!$A$1:$M$9</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'Project_Content'!$A$1:$L$9</definedName>
@@ -540,12 +540,12 @@
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>Safety</t>
+          <t>Public contact</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>API에는 개인 전화번호, 비공개 이메일, 자격증 번호를 공개하지 마세요.</t>
+          <t>API에는 khkim1729@gmail.com과 자격증 번호를 공개합니다. 개인 전화번호는 입력하지 않습니다.</t>
         </is>
       </c>
     </row>
@@ -1759,12 +1759,12 @@
       </c>
       <c r="J1" s="1" t="inlineStr">
         <is>
-          <t>credential_number_private</t>
+          <t>credential_number</t>
         </is>
       </c>
       <c r="K1" s="1" t="inlineStr">
         <is>
-          <t>credential_id_private</t>
+          <t>verification_id</t>
         </is>
       </c>
       <c r="L1" s="1" t="inlineStr">
@@ -3400,7 +3400,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Apps Script allowlist에 포함된 공개 열만 반환합니다. *_private 열은 절대 반환하지 않습니다.</t>
+          <t>공개 이메일과 credential_number/verification_id를 반환합니다. 개인 전화번호 열은 만들거나 입력하지 않습니다.</t>
         </is>
       </c>
     </row>
@@ -3440,7 +3440,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E7"/>
+  <dimension ref="A1:E8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -3627,8 +3627,35 @@
       </c>
       <c r="E7" s="2" t="inlineStr"/>
     </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>public_email</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>khkim1729@gmail.com</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>khkim1729@gmail.com</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>Public contact email; do not add a phone number.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:E7"/>
+  <autoFilter ref="A1:E8"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -23189,14 +23216,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X2"/>
+  <dimension ref="A1:X44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
     <col width="18" customWidth="1" min="2" max="2"/>
-    <col width="18" customWidth="1" min="3" max="3"/>
-    <col width="18" customWidth="1" min="4" max="4"/>
-    <col width="18" customWidth="1" min="5" max="5"/>
+    <col width="55" customWidth="1" min="3" max="3"/>
+    <col width="42" customWidth="1" min="4" max="4"/>
+    <col width="70" customWidth="1" min="5" max="5"/>
     <col width="18" customWidth="1" min="6" max="6"/>
     <col width="18" customWidth="1" min="7" max="7"/>
     <col width="18" customWidth="1" min="8" max="8"/>
@@ -23341,13 +23368,3561 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2">
-        <f>ARRAYFORMULA(IF(DB_Publications!A2:A="","",DB_Publications!A2:X))</f>
-        <v/>
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>KHK_UR_010</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="n">
+        <v>2027</v>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>HERO: Hybrid PET-CT Representation Learning for Head and Neck Tumor Segmentation and Outcome Prediction</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>AAAI 2027</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>Kyeonghun Kim, Minju Kim, Tae Gyun Kim, Juyeon Yoo, Yehee Kim, Seohyeon Ji, Seokjun Choi, Kyung Seok Yuh, Pa Hong, Ken Ying-Kai Liao, Nam-Joon Kim†</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr"/>
+      <c r="G2" s="2" t="inlineStr"/>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>Under review</t>
+        </is>
+      </c>
+      <c r="I2" s="2" t="inlineStr"/>
+      <c r="J2" s="2" t="inlineStr"/>
+      <c r="K2" s="2" t="inlineStr"/>
+      <c r="L2" s="2" t="inlineStr"/>
+      <c r="M2" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="N2" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="O2" s="2" t="inlineStr">
+        <is>
+          <t>Under Review</t>
+        </is>
+      </c>
+      <c r="P2" s="2" t="inlineStr">
+        <is>
+          <t>Conference</t>
+        </is>
+      </c>
+      <c r="Q2" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="R2" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="S2" s="2" t="n">
+        <v>430</v>
+      </c>
+      <c r="T2" s="2" t="inlineStr"/>
+      <c r="U2" s="2" t="inlineStr"/>
+      <c r="V2" s="2" t="inlineStr">
+        <is>
+          <t>심사 중</t>
+        </is>
+      </c>
+      <c r="W2" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="X2" s="2" t="inlineStr">
+        <is>
+          <t>Personal</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>KHK_UR_009</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="n">
+        <v>2027</v>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>SSDenoDet: Self-Supervised Cross-Domain Feature Denoising for SAR Target Detection</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>AAAI 2027</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>Kyeonghun Kim, Yului Jeong, Youngung Han, Yunjin Seo, Youngseo Kim, Yeonghyeon Park, SeoJeong Woo, Giseong Hwang, Ken Ying-Kai Liao, Nam-Joon Kim†</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr"/>
+      <c r="G3" s="2" t="inlineStr"/>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>Under review</t>
+        </is>
+      </c>
+      <c r="I3" s="2" t="inlineStr"/>
+      <c r="J3" s="2" t="inlineStr"/>
+      <c r="K3" s="2" t="inlineStr"/>
+      <c r="L3" s="2" t="inlineStr"/>
+      <c r="M3" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="N3" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="O3" s="2" t="inlineStr">
+        <is>
+          <t>Under Review</t>
+        </is>
+      </c>
+      <c r="P3" s="2" t="inlineStr">
+        <is>
+          <t>Conference</t>
+        </is>
+      </c>
+      <c r="Q3" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="R3" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="S3" s="2" t="n">
+        <v>420</v>
+      </c>
+      <c r="T3" s="2" t="inlineStr"/>
+      <c r="U3" s="2" t="inlineStr"/>
+      <c r="V3" s="2" t="inlineStr">
+        <is>
+          <t>심사 중</t>
+        </is>
+      </c>
+      <c r="W3" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="X3" s="2" t="inlineStr">
+        <is>
+          <t>Personal</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>KHK_UR_008</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>Hierarchy Aware Preference Optimization for the Safety of Korean Small Language Models</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>EMNLP 2026</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>Soo Yong Kim, Junyoung Koh, Kyeonghun Kim, Seunghyeok Hong†</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr"/>
+      <c r="G4" s="2" t="inlineStr"/>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
+          <t>Under review</t>
+        </is>
+      </c>
+      <c r="I4" s="2" t="inlineStr"/>
+      <c r="J4" s="2" t="inlineStr"/>
+      <c r="K4" s="2" t="inlineStr"/>
+      <c r="L4" s="2" t="inlineStr"/>
+      <c r="M4" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="N4" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="O4" s="2" t="inlineStr">
+        <is>
+          <t>Under Review</t>
+        </is>
+      </c>
+      <c r="P4" s="2" t="inlineStr">
+        <is>
+          <t>Conference</t>
+        </is>
+      </c>
+      <c r="Q4" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="R4" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="S4" s="2" t="n">
+        <v>410</v>
+      </c>
+      <c r="T4" s="2" t="inlineStr"/>
+      <c r="U4" s="2" t="inlineStr"/>
+      <c r="V4" s="2" t="inlineStr">
+        <is>
+          <t>심사 중</t>
+        </is>
+      </c>
+      <c r="W4" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="X4" s="2" t="inlineStr">
+        <is>
+          <t>Personal</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>KHK_UR_007</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="n">
+        <v>2027</v>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>Period Deserts: Controlled Corpus Interventions Induce and Repair Forecasting Failures in Time-Series Models</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>AAAI 2027</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>Eunseob Choi, Kyeonghun Kim, Hyuk-Jae Lee, Nam-Joon Kim†</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr"/>
+      <c r="G5" s="2" t="inlineStr"/>
+      <c r="H5" s="2" t="inlineStr">
+        <is>
+          <t>Under review</t>
+        </is>
+      </c>
+      <c r="I5" s="2" t="inlineStr"/>
+      <c r="J5" s="2" t="inlineStr"/>
+      <c r="K5" s="2" t="inlineStr"/>
+      <c r="L5" s="2" t="inlineStr"/>
+      <c r="M5" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="N5" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="O5" s="2" t="inlineStr">
+        <is>
+          <t>Under Review</t>
+        </is>
+      </c>
+      <c r="P5" s="2" t="inlineStr">
+        <is>
+          <t>Conference</t>
+        </is>
+      </c>
+      <c r="Q5" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="R5" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="S5" s="2" t="n">
+        <v>400</v>
+      </c>
+      <c r="T5" s="2" t="inlineStr"/>
+      <c r="U5" s="2" t="inlineStr"/>
+      <c r="V5" s="2" t="inlineStr">
+        <is>
+          <t>심사 중</t>
+        </is>
+      </c>
+      <c r="W5" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="X5" s="2" t="inlineStr">
+        <is>
+          <t>Personal</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>KHK_UR_006</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="n">
+        <v>2027</v>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>QDDPM: Quaternion Denoising Diffusion Probabilistic Models for Zero-Cost Super-Resolution</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>AAAI 2027</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>Seongheon Choi, Kyeonghun Kim, Insung Hwang, Taeyun Kim, Donghyeon Seo, Suemin Yang, Yoonseon Jung, Seoyoon Koo, Wonhyuk Kim, Pa Hong, Ken Ying-Kai Liao, Hyuk-Jae Lee, Nam-Joon Kim†</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr"/>
+      <c r="G6" s="2" t="inlineStr"/>
+      <c r="H6" s="2" t="inlineStr">
+        <is>
+          <t>Under review</t>
+        </is>
+      </c>
+      <c r="I6" s="2" t="inlineStr"/>
+      <c r="J6" s="2" t="inlineStr"/>
+      <c r="K6" s="2" t="inlineStr"/>
+      <c r="L6" s="2" t="inlineStr"/>
+      <c r="M6" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="N6" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="O6" s="2" t="inlineStr">
+        <is>
+          <t>Under Review</t>
+        </is>
+      </c>
+      <c r="P6" s="2" t="inlineStr">
+        <is>
+          <t>Conference</t>
+        </is>
+      </c>
+      <c r="Q6" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="R6" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="S6" s="2" t="n">
+        <v>390</v>
+      </c>
+      <c r="T6" s="2" t="inlineStr"/>
+      <c r="U6" s="2" t="inlineStr"/>
+      <c r="V6" s="2" t="inlineStr">
+        <is>
+          <t>심사 중</t>
+        </is>
+      </c>
+      <c r="W6" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="X6" s="2" t="inlineStr">
+        <is>
+          <t>Personal</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>KHK_UR_005</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="n">
+        <v>2027</v>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>FBI: A Framework for Benchmark Integrity via Keyed Option-Order Fingerprinting</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>AAAI 2027</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>Ina Jung, Kyeonghun Kim, Youngung Han, Seungwoo Baek, Jiwon Park, Minjeong Kim, Minseo Kim, Soo Yong Kim, Je Won Yeom, Sieun Hyeon†</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="inlineStr"/>
+      <c r="G7" s="2" t="inlineStr"/>
+      <c r="H7" s="2" t="inlineStr">
+        <is>
+          <t>Under review</t>
+        </is>
+      </c>
+      <c r="I7" s="2" t="inlineStr"/>
+      <c r="J7" s="2" t="inlineStr"/>
+      <c r="K7" s="2" t="inlineStr"/>
+      <c r="L7" s="2" t="inlineStr"/>
+      <c r="M7" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="N7" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="O7" s="2" t="inlineStr">
+        <is>
+          <t>Under Review</t>
+        </is>
+      </c>
+      <c r="P7" s="2" t="inlineStr">
+        <is>
+          <t>Conference</t>
+        </is>
+      </c>
+      <c r="Q7" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="R7" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="S7" s="2" t="n">
+        <v>380</v>
+      </c>
+      <c r="T7" s="2" t="inlineStr"/>
+      <c r="U7" s="2" t="inlineStr"/>
+      <c r="V7" s="2" t="inlineStr">
+        <is>
+          <t>심사 중</t>
+        </is>
+      </c>
+      <c r="W7" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="X7" s="2" t="inlineStr">
+        <is>
+          <t>Personal</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>KHK_UR_004</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>Auditing Capsule Vision 2024: Within-Split Train-to-Validation Re-Exposure and a Kvasir-Channel Sensitivity Diagnostic</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>NeurIPS 2026</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>Eunseob Choi, Kyeonghun Kim, Hyuk-Jae Lee, Nam-Joon Kim†</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="inlineStr"/>
+      <c r="G8" s="2" t="inlineStr"/>
+      <c r="H8" s="2" t="inlineStr">
+        <is>
+          <t>Under review</t>
+        </is>
+      </c>
+      <c r="I8" s="2" t="inlineStr"/>
+      <c r="J8" s="2" t="inlineStr"/>
+      <c r="K8" s="2" t="inlineStr"/>
+      <c r="L8" s="2" t="inlineStr"/>
+      <c r="M8" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="N8" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="O8" s="2" t="inlineStr">
+        <is>
+          <t>Under Review</t>
+        </is>
+      </c>
+      <c r="P8" s="2" t="inlineStr">
+        <is>
+          <t>Conference</t>
+        </is>
+      </c>
+      <c r="Q8" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="R8" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="S8" s="2" t="n">
+        <v>370</v>
+      </c>
+      <c r="T8" s="2" t="inlineStr"/>
+      <c r="U8" s="2" t="inlineStr"/>
+      <c r="V8" s="2" t="inlineStr">
+        <is>
+          <t>심사 중</t>
+        </is>
+      </c>
+      <c r="W8" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="X8" s="2" t="inlineStr">
+        <is>
+          <t>Personal</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>KHK_UR_003</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>Auditing Correlated Failures in Frozen-Feature Pretrained-Encoder Pools for Medical Segmentation</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>NeurIPS 2026</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>Eunseob Choi, Kyeonghun Kim, Hyuk-Jae Lee, Nam-Joon Kim†</t>
+        </is>
+      </c>
+      <c r="F9" s="2" t="inlineStr"/>
+      <c r="G9" s="2" t="inlineStr"/>
+      <c r="H9" s="2" t="inlineStr">
+        <is>
+          <t>Under review</t>
+        </is>
+      </c>
+      <c r="I9" s="2" t="inlineStr"/>
+      <c r="J9" s="2" t="inlineStr"/>
+      <c r="K9" s="2" t="inlineStr"/>
+      <c r="L9" s="2" t="inlineStr"/>
+      <c r="M9" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="N9" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="O9" s="2" t="inlineStr">
+        <is>
+          <t>Under Review</t>
+        </is>
+      </c>
+      <c r="P9" s="2" t="inlineStr">
+        <is>
+          <t>Conference</t>
+        </is>
+      </c>
+      <c r="Q9" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="R9" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="S9" s="2" t="n">
+        <v>360</v>
+      </c>
+      <c r="T9" s="2" t="inlineStr"/>
+      <c r="U9" s="2" t="inlineStr"/>
+      <c r="V9" s="2" t="inlineStr">
+        <is>
+          <t>심사 중</t>
+        </is>
+      </c>
+      <c r="W9" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="X9" s="2" t="inlineStr">
+        <is>
+          <t>Personal</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>KHK_UR_002</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>Task-Side Geometry Shapes Terminal Class Geometry</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>NeurIPS 2026</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>Minseo Choi, Youngung Han, Kyeonghun Kim, Yoohyun Kim, Jewoo Park, Seungwon Park, Seoyoung Ju, Ken Ying-Kai Liao, Hyuk-Jae Lee, Nam-Joon Kim†</t>
+        </is>
+      </c>
+      <c r="F10" s="2" t="inlineStr"/>
+      <c r="G10" s="2" t="inlineStr"/>
+      <c r="H10" s="2" t="inlineStr">
+        <is>
+          <t>Under review</t>
+        </is>
+      </c>
+      <c r="I10" s="2" t="inlineStr"/>
+      <c r="J10" s="2" t="inlineStr"/>
+      <c r="K10" s="2" t="inlineStr"/>
+      <c r="L10" s="2" t="inlineStr"/>
+      <c r="M10" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="N10" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="O10" s="2" t="inlineStr">
+        <is>
+          <t>Under Review</t>
+        </is>
+      </c>
+      <c r="P10" s="2" t="inlineStr">
+        <is>
+          <t>Conference</t>
+        </is>
+      </c>
+      <c r="Q10" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="R10" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="S10" s="2" t="n">
+        <v>350</v>
+      </c>
+      <c r="T10" s="2" t="inlineStr"/>
+      <c r="U10" s="2" t="inlineStr"/>
+      <c r="V10" s="2" t="inlineStr">
+        <is>
+          <t>심사 중</t>
+        </is>
+      </c>
+      <c r="W10" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="X10" s="2" t="inlineStr">
+        <is>
+          <t>Personal</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>KHK_UR_001</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>Automated dental caries segmentation in panoramic radiographs using a lightweight dual-stage deep learning framework</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>Scientific Reports</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>Yeongseok Seo, Kyeonghun Kim, Jong-yeol Lee, Jihun Kim, Dohyun Chun†</t>
+        </is>
+      </c>
+      <c r="F11" s="2" t="inlineStr"/>
+      <c r="G11" s="2" t="inlineStr"/>
+      <c r="H11" s="2" t="inlineStr">
+        <is>
+          <t>Under review</t>
+        </is>
+      </c>
+      <c r="I11" s="2" t="inlineStr"/>
+      <c r="J11" s="2" t="inlineStr"/>
+      <c r="K11" s="2" t="inlineStr"/>
+      <c r="L11" s="2" t="inlineStr"/>
+      <c r="M11" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="N11" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="O11" s="2" t="inlineStr">
+        <is>
+          <t>Under Review</t>
+        </is>
+      </c>
+      <c r="P11" s="2" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="Q11" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="R11" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="S11" s="2" t="n">
+        <v>340</v>
+      </c>
+      <c r="T11" s="2" t="inlineStr"/>
+      <c r="U11" s="2" t="inlineStr"/>
+      <c r="V11" s="2" t="inlineStr">
+        <is>
+          <t>심사 중</t>
+        </is>
+      </c>
+      <c r="W11" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="X11" s="2" t="inlineStr">
+        <is>
+          <t>Personal</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>PUB_053</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>PANDA: Phase-Aware Network with Diffusion Refinement and Expert Aggregation for PNI Detection in Multi-phase MRI</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>Proceedings of the 41st Annual AAAI Conference on Artificial Intelligence (AAAI) (Under Review)</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>Youngung Han, Dohyun Kweon, Kyeonghun Kim, Hyunsu Go, Junga Kim, Induk Um, Jaewon Jung, Jina Jeong, Anna Jung, Minjae Park, Woo Kyoung Jeong, Won Jae Lee, Pa Hong, Ping Shu Ho, Tak Shing Au Yeung, Ka Chun Cheung, Ken Ying-Kai Liao, Hyuk-Jae Lee, Nam-Joon Kim†</t>
+        </is>
+      </c>
+      <c r="F12" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G12" s="2" t="inlineStr">
+        <is>
+          <t>https://aaai.org/conference/aaai/aaai-27/</t>
+        </is>
+      </c>
+      <c r="H12" s="2" t="inlineStr"/>
+      <c r="I12" s="2" t="inlineStr"/>
+      <c r="J12" s="2" t="inlineStr"/>
+      <c r="K12" s="2" t="inlineStr"/>
+      <c r="L12" s="2" t="inlineStr"/>
+      <c r="M12" s="2" t="inlineStr"/>
+      <c r="N12" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="O12" s="2" t="inlineStr">
+        <is>
+          <t>Under Review</t>
+        </is>
+      </c>
+      <c r="P12" s="2" t="inlineStr">
+        <is>
+          <t>Conference</t>
+        </is>
+      </c>
+      <c r="Q12" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="R12" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="S12" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="T12" s="2" t="inlineStr"/>
+      <c r="U12" s="2" t="inlineStr"/>
+      <c r="V12" s="2" t="inlineStr"/>
+      <c r="W12" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="X12" s="2" t="inlineStr">
+        <is>
+          <t>IMSI WEB_Publications</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>PUB_052</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>State-Space Modeling of Spatial Structure and Phase Dynamics for Perineural Invasion Prediction in Multi-Phase 3D MRI</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>Proceedings of the 41st Annual AAAI Conference on Artificial Intelligence (AAAI) (Under Review)</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr">
+        <is>
+          <t>Youngung Han, Hyunsu Go, Kyeonghun Kim, Induk Um, Junga Kim, Dohyun Kweon, Jaewon Jung, Jina Jeong, Sungha Park, Minjae Park, Woo Kyoung Jeong, Won Jae Lee, Pa Hong, Ping Shu Ho, Tak Shing Au Yeung, Ka Chun Cheung, Ken Ying-Kai Liao, Hyuk-Jae Lee, Nam-Joon Kim†</t>
+        </is>
+      </c>
+      <c r="F13" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G13" s="2" t="inlineStr">
+        <is>
+          <t>https://aaai.org/conference/aaai/aaai-27/</t>
+        </is>
+      </c>
+      <c r="H13" s="2" t="inlineStr"/>
+      <c r="I13" s="2" t="inlineStr"/>
+      <c r="J13" s="2" t="inlineStr"/>
+      <c r="K13" s="2" t="inlineStr"/>
+      <c r="L13" s="2" t="inlineStr"/>
+      <c r="M13" s="2" t="inlineStr"/>
+      <c r="N13" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="O13" s="2" t="inlineStr">
+        <is>
+          <t>Under Review</t>
+        </is>
+      </c>
+      <c r="P13" s="2" t="inlineStr">
+        <is>
+          <t>Conference</t>
+        </is>
+      </c>
+      <c r="Q13" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="R13" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="S13" s="2" t="n">
+        <v>40</v>
+      </c>
+      <c r="T13" s="2" t="inlineStr"/>
+      <c r="U13" s="2" t="inlineStr"/>
+      <c r="V13" s="2" t="inlineStr"/>
+      <c r="W13" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="X13" s="2" t="inlineStr">
+        <is>
+          <t>IMSI WEB_Publications</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>PUB_051</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>MAESTRO: Multi-phase Adaptive Experts with Spiking Temporal-spatial Routing Network for Perineural Invasion Prediction in 3D MRI</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>Proceedings of the 41st Annual AAAI Conference on Artificial Intelligence (AAAI) (Under Review)</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>Youngung Han, Induk Um, Kyeonghun Kim, Hyunsu Go, Junga Kim, Dohyun Kweon, Jaewon Jung, Jina Jeong, Yuluei Jeong, Minjae Park, Woo Kyoung Jeong, Won Jae Lee, Pa Hong, Ping Shu Ho, Tak Shing Au Yeung, Ka Chun Cheung, Ken Ying-Kai Liao, Hyuk-Jae Lee, Nam-Joon Kim†</t>
+        </is>
+      </c>
+      <c r="F14" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G14" s="2" t="inlineStr">
+        <is>
+          <t>https://aaai.org/conference/aaai/aaai-27/</t>
+        </is>
+      </c>
+      <c r="H14" s="2" t="inlineStr"/>
+      <c r="I14" s="2" t="inlineStr"/>
+      <c r="J14" s="2" t="inlineStr"/>
+      <c r="K14" s="2" t="inlineStr"/>
+      <c r="L14" s="2" t="inlineStr"/>
+      <c r="M14" s="2" t="inlineStr"/>
+      <c r="N14" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="O14" s="2" t="inlineStr">
+        <is>
+          <t>Under Review</t>
+        </is>
+      </c>
+      <c r="P14" s="2" t="inlineStr">
+        <is>
+          <t>Conference</t>
+        </is>
+      </c>
+      <c r="Q14" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="R14" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="S14" s="2" t="n">
+        <v>50</v>
+      </c>
+      <c r="T14" s="2" t="inlineStr"/>
+      <c r="U14" s="2" t="inlineStr"/>
+      <c r="V14" s="2" t="inlineStr"/>
+      <c r="W14" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="X14" s="2" t="inlineStr">
+        <is>
+          <t>IMSI WEB_Publications</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>PUB_050</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>FiLMamba: FiLM-Conditioned State Space Models for 3D Multi-Coil MRI Reconstruction</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>Proceedings of the 41st Annual AAAI Conference on Artificial Intelligence (AAAI) (Under Review)</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="inlineStr">
+        <is>
+          <t>Eunseob Choi, Hyeonseok Jung, Kyeonghun Kim, Pa Hong, Hyuk-Jae Lee, Nam-Joon Kim†</t>
+        </is>
+      </c>
+      <c r="F15" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G15" s="2" t="inlineStr">
+        <is>
+          <t>https://aaai.org/conference/aaai/aaai-27/</t>
+        </is>
+      </c>
+      <c r="H15" s="2" t="inlineStr"/>
+      <c r="I15" s="2" t="inlineStr"/>
+      <c r="J15" s="2" t="inlineStr"/>
+      <c r="K15" s="2" t="inlineStr"/>
+      <c r="L15" s="2" t="inlineStr"/>
+      <c r="M15" s="2" t="inlineStr"/>
+      <c r="N15" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="O15" s="2" t="inlineStr">
+        <is>
+          <t>Under Review</t>
+        </is>
+      </c>
+      <c r="P15" s="2" t="inlineStr">
+        <is>
+          <t>Conference</t>
+        </is>
+      </c>
+      <c r="Q15" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="R15" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="S15" s="2" t="n">
+        <v>60</v>
+      </c>
+      <c r="T15" s="2" t="inlineStr"/>
+      <c r="U15" s="2" t="inlineStr"/>
+      <c r="V15" s="2" t="inlineStr"/>
+      <c r="W15" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="X15" s="2" t="inlineStr">
+        <is>
+          <t>IMSI WEB_Publications</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>PUB_049</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>MATHENA: Mamba-based Architectural Tooth Hierarchical Estimator and Holistic Evaluation Network for Anatomy</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>The 18th Asian Conference on Computer Vision (ACCV 2026) (Under Review)</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t>Kyeonghun Kim, Jaehyung Park, Youngung Han, Anna Jung, Seongbin Park, Sumin Lee, Jiwon Yang, Jiyoon Han, Subeen Lee, Junsu Lim, Hyunsu Go, Eunseob Choi, Hyeonseok Jung, Soo Yong Kim, Woo Kyoung Jeong, Won Jae Lee, Pa Hong, Ken Ying-Kai Liao, Hyuk-Jae Lee, Nam-Joon Kim†</t>
+        </is>
+      </c>
+      <c r="F16" s="2" t="inlineStr">
+        <is>
+          <t>https://arxiv.org/abs/2604.00537</t>
+        </is>
+      </c>
+      <c r="G16" s="2" t="inlineStr">
+        <is>
+          <t>https://accv2026.org/</t>
+        </is>
+      </c>
+      <c r="H16" s="2" t="inlineStr"/>
+      <c r="I16" s="2" t="inlineStr">
+        <is>
+          <t>https://github.com/khkim1729/mathena</t>
+        </is>
+      </c>
+      <c r="J16" s="2" t="inlineStr"/>
+      <c r="K16" s="2" t="inlineStr"/>
+      <c r="L16" s="2" t="inlineStr">
+        <is>
+          <t>@article{kim2026mathena,
+  title={MATHENA: Mamba-based Architectural Tooth Hierarchical Estimator and Holistic Evaluation Network for Anatomy},
+  author={Kim, Kyeonghun and Park, Jaehyung and Han, Youngung and Jung, Anna and Park, Seongbin and Lee, Sumin and Yang, Jiwon and Han, Jiyoon and Lee, Subeen and Lim, Junsu and others},
+  journal={arXiv preprint arXiv:2604.00537},
+  year={2026}
+}</t>
+        </is>
+      </c>
+      <c r="M16" s="2" t="inlineStr"/>
+      <c r="N16" s="2" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="O16" s="2" t="inlineStr">
+        <is>
+          <t>Under Review</t>
+        </is>
+      </c>
+      <c r="P16" s="2" t="inlineStr">
+        <is>
+          <t>Conference</t>
+        </is>
+      </c>
+      <c r="Q16" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="R16" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="S16" s="2" t="n">
+        <v>70</v>
+      </c>
+      <c r="T16" s="2" t="inlineStr"/>
+      <c r="U16" s="2" t="inlineStr"/>
+      <c r="V16" s="2" t="inlineStr"/>
+      <c r="W16" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="X16" s="2" t="inlineStr">
+        <is>
+          <t>IMSI WEB_Publications</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>PUB_048</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>NEMESIS: Noise-suppressed Efficient MAE with Enhanced Superpatch Integration Strategy</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>The 18th Asian Conference on Computer Vision (ACCV 2026) (Under Review)</t>
+        </is>
+      </c>
+      <c r="E17" s="2" t="inlineStr">
+        <is>
+          <t>Kyeonghun Kim, Hyeonseok Jung, Youngung Han, Hyunsu Go, Eunseob Choi, Seongbin Park, Junsu Lim, Jiwon Yang, Sumin Lee, Ken Ying-Kai Liao, Nam-Joon Kim†</t>
+        </is>
+      </c>
+      <c r="F17" s="2" t="inlineStr">
+        <is>
+          <t>https://arxiv.org/abs/2604.01612</t>
+        </is>
+      </c>
+      <c r="G17" s="2" t="inlineStr">
+        <is>
+          <t>https://accv2026.org/</t>
+        </is>
+      </c>
+      <c r="H17" s="2" t="inlineStr"/>
+      <c r="I17" s="2" t="inlineStr"/>
+      <c r="J17" s="2" t="inlineStr"/>
+      <c r="K17" s="2" t="inlineStr"/>
+      <c r="L17" s="2" t="inlineStr">
+        <is>
+          <t>@article{kim2026nemesis,
+  title={NEMESIS: Noise-suppressed Efficient MAE with Enhanced Superpatch Integration Strategy},
+  author={Kim, Kyeonghun and Jung, Hyeonseok and Han, Youngung and Go, Hyunsu and Choi, Eunseob and Park, Seongbin and Lim, Junsu and Yang, Jiwon and Lee, Sumin and Hwang, Insung and others},
+  journal={arXiv preprint arXiv:2604.01612},
+  year={2026}
+}</t>
+        </is>
+      </c>
+      <c r="M17" s="2" t="inlineStr"/>
+      <c r="N17" s="2" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="O17" s="2" t="inlineStr">
+        <is>
+          <t>Under Review</t>
+        </is>
+      </c>
+      <c r="P17" s="2" t="inlineStr">
+        <is>
+          <t>Conference</t>
+        </is>
+      </c>
+      <c r="Q17" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="R17" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="S17" s="2" t="n">
+        <v>80</v>
+      </c>
+      <c r="T17" s="2" t="inlineStr"/>
+      <c r="U17" s="2" t="inlineStr"/>
+      <c r="V17" s="2" t="inlineStr"/>
+      <c r="W17" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="X17" s="2" t="inlineStr">
+        <is>
+          <t>IMSI WEB_Publications</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>PUB_047</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>TIME: 2.5D IDH-predictive Multimodal Ensemble for multitask glioma subtypin</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>The 18th Asian Conference on Computer Vision (ACCV 2026) (Under Review)</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="inlineStr">
+        <is>
+          <t>Kyeonghun Kim, Jieon Kim, Seongheon Choi, Donghyeon Seo, Minchan Kim, Insung Hwang, Suemin Yang , Taeyun Kim, Seoyoon Koo , Wonhyuk Kim, Yoonseon Jung, Woo Kyoung Jeong, Won Jae Lee, Pa Hong, Ken Ying-Kai Liao, Hyuk-Jae Lee, Nam-Joon Kim†</t>
+        </is>
+      </c>
+      <c r="F18" s="2" t="inlineStr">
+        <is>
+          <t>https://drive.google.com/file/d/1fDHV8Q5YXQC9s_mfPZ09AkOPoF_YWgyg/view?usp=sharing</t>
+        </is>
+      </c>
+      <c r="G18" s="2" t="inlineStr">
+        <is>
+          <t>https://accv2026.org/</t>
+        </is>
+      </c>
+      <c r="H18" s="2" t="inlineStr"/>
+      <c r="I18" s="2" t="inlineStr">
+        <is>
+          <t>https://github.com/khkim1729/TIME</t>
+        </is>
+      </c>
+      <c r="J18" s="2" t="inlineStr"/>
+      <c r="K18" s="2" t="inlineStr"/>
+      <c r="L18" s="2" t="inlineStr"/>
+      <c r="M18" s="2" t="inlineStr"/>
+      <c r="N18" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="O18" s="2" t="inlineStr">
+        <is>
+          <t>Under Review</t>
+        </is>
+      </c>
+      <c r="P18" s="2" t="inlineStr">
+        <is>
+          <t>Conference</t>
+        </is>
+      </c>
+      <c r="Q18" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="R18" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="S18" s="2" t="n">
+        <v>90</v>
+      </c>
+      <c r="T18" s="2" t="inlineStr"/>
+      <c r="U18" s="2" t="inlineStr"/>
+      <c r="V18" s="2" t="inlineStr"/>
+      <c r="W18" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="X18" s="2" t="inlineStr">
+        <is>
+          <t>IMSI WEB_Publications</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>PUB_046</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t>DICE: 2.5D DINOv2-Based IDH-Centric Cascaded Embedding Model for Integrated Glioma Diagnosis</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="inlineStr">
+        <is>
+          <t>The 18th Asian Conference on Computer Vision (ACCV 2026) (Under Review)</t>
+        </is>
+      </c>
+      <c r="E19" s="2" t="inlineStr">
+        <is>
+          <t>Seongheon Choi, Kyeonghun Kim, Jieon Kim, Donghyeon Seo, Minchan Kim, Insung Hwang, Suemin Yang, Taeyun Kim, Yoonseon Jung, Wonhyuk Kim, Seoyoon Koo, Pa Hong, Ken Ying-Kai Liao, Hyuk-Jae Lee, Nam-Joon Kim†</t>
+        </is>
+      </c>
+      <c r="F19" s="2" t="inlineStr">
+        <is>
+          <t>https://drive.google.com/file/d/1kHtrykQuD1RE-CnOR_xyoAgQBKK6w5Qi/view?usp=sharing</t>
+        </is>
+      </c>
+      <c r="G19" s="2" t="inlineStr">
+        <is>
+          <t>https://accv2026.org/</t>
+        </is>
+      </c>
+      <c r="H19" s="2" t="inlineStr"/>
+      <c r="I19" s="2" t="inlineStr"/>
+      <c r="J19" s="2" t="inlineStr"/>
+      <c r="K19" s="2" t="inlineStr"/>
+      <c r="L19" s="2" t="inlineStr"/>
+      <c r="M19" s="2" t="inlineStr"/>
+      <c r="N19" s="2" t="inlineStr"/>
+      <c r="O19" s="2" t="inlineStr">
+        <is>
+          <t>Under Review</t>
+        </is>
+      </c>
+      <c r="P19" s="2" t="inlineStr">
+        <is>
+          <t>Conference</t>
+        </is>
+      </c>
+      <c r="Q19" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="R19" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="S19" s="2" t="n">
+        <v>100</v>
+      </c>
+      <c r="T19" s="2" t="inlineStr"/>
+      <c r="U19" s="2" t="inlineStr"/>
+      <c r="V19" s="2" t="inlineStr"/>
+      <c r="W19" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="X19" s="2" t="inlineStr">
+        <is>
+          <t>IMSI WEB_Publications</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>PUB_045</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t>LeafFireNet: Hyperspectral Leaf Dryness Classification for Wildfire Risk Prediction Using Temporal SWIR Spectral Signatures</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="inlineStr">
+        <is>
+          <t>IEIE 2026 Summer (대한전자공학회 하계학술대회), 2026</t>
+        </is>
+      </c>
+      <c r="E20" s="2" t="inlineStr">
+        <is>
+          <t>Insung Hwang, Kyeonghun Kim, Youngung Han, Eunseob Choi, Tien Nguyen, Sumin Lee, Subeen Lee, Anna Jung, Jiwon Yang, Hyeonseok Jung, Junsu Lim, Hyunsu Go, Seongbin Park, Ken Ying-Kai Liao, Nam-Joon Kim†</t>
+        </is>
+      </c>
+      <c r="F20" s="2" t="inlineStr">
+        <is>
+          <t>https://drive.google.com/file/d/1CeU2YtiGSEiZpesBosrizRQ9cJPoXySR/view?usp=drive_link</t>
+        </is>
+      </c>
+      <c r="G20" s="2" t="inlineStr">
+        <is>
+          <t>https://conf.theieie.org/2026s/</t>
+        </is>
+      </c>
+      <c r="H20" s="2" t="inlineStr"/>
+      <c r="I20" s="2" t="inlineStr"/>
+      <c r="J20" s="2" t="inlineStr"/>
+      <c r="K20" s="2" t="inlineStr"/>
+      <c r="L20" s="2" t="inlineStr"/>
+      <c r="M20" s="2" t="inlineStr"/>
+      <c r="N20" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="O20" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="P20" s="2" t="inlineStr">
+        <is>
+          <t>Conference</t>
+        </is>
+      </c>
+      <c r="Q20" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="R20" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="S20" s="2" t="n">
+        <v>110</v>
+      </c>
+      <c r="T20" s="2" t="inlineStr"/>
+      <c r="U20" s="2" t="inlineStr"/>
+      <c r="V20" s="2" t="inlineStr"/>
+      <c r="W20" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="X20" s="2" t="inlineStr">
+        <is>
+          <t>IMSI WEB_Publications</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>PUB_044</t>
+        </is>
+      </c>
+      <c r="B21" s="2" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C21" s="2" t="inlineStr">
+        <is>
+          <t>DAPP: Deep Learning Architecture for Predicting Pathological Characteristics of Gliomas Based on Multi-Medical Data Fusion</t>
+        </is>
+      </c>
+      <c r="D21" s="2" t="inlineStr">
+        <is>
+          <t>IEIE 2026 Summer (대한전자공학회 하계학술대회), 2026</t>
+        </is>
+      </c>
+      <c r="E21" s="2" t="inlineStr">
+        <is>
+          <t>Suemin Yang, Seongheon Choi, Kyeonghun Kim, Insung Hwang,  Donghyeon Seo, Minchan Kim, Seoyoon Koo, Taeyun Kim, Yoonseon Jung, Wonhyuk Kim, Ken Ying-Kai Liao, Nam-Joon Kim†</t>
+        </is>
+      </c>
+      <c r="F21" s="2" t="inlineStr">
+        <is>
+          <t>https://drive.google.com/file/d/1lZD70gbZfovR3DywSeJji7MJzimucpy9/view?usp=sharing</t>
+        </is>
+      </c>
+      <c r="G21" s="2" t="inlineStr">
+        <is>
+          <t>https://conf.theieie.org/2026s/</t>
+        </is>
+      </c>
+      <c r="H21" s="2" t="inlineStr"/>
+      <c r="I21" s="2" t="inlineStr"/>
+      <c r="J21" s="2" t="inlineStr"/>
+      <c r="K21" s="2" t="inlineStr"/>
+      <c r="L21" s="2" t="inlineStr"/>
+      <c r="M21" s="2" t="inlineStr"/>
+      <c r="N21" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="O21" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="P21" s="2" t="inlineStr">
+        <is>
+          <t>Conference</t>
+        </is>
+      </c>
+      <c r="Q21" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="R21" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="S21" s="2" t="n">
+        <v>120</v>
+      </c>
+      <c r="T21" s="2" t="inlineStr"/>
+      <c r="U21" s="2" t="inlineStr"/>
+      <c r="V21" s="2" t="inlineStr"/>
+      <c r="W21" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="X21" s="2" t="inlineStr">
+        <is>
+          <t>IMSI WEB_Publications</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>PUB_043</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t>FUMM: Feasibility of Using Multiple Modalities for Prostate Cancer Classification and Grading</t>
+        </is>
+      </c>
+      <c r="D22" s="2" t="inlineStr">
+        <is>
+          <t>IEIE 2026 Summer (대한전자공학회 하계학술대회), 2026</t>
+        </is>
+      </c>
+      <c r="E22" s="2" t="inlineStr">
+        <is>
+          <t>Anna Jung, Kyeonghun Kim, Youngung Han, Ken Ying-Kai Liao, Nam-Joon Kim†</t>
+        </is>
+      </c>
+      <c r="F22" s="2" t="inlineStr">
+        <is>
+          <t>https://drive.google.com/file/d/1O684gvMbNtSsJWDX5_ZqfhjEl_63tLtc/view?usp=drive_link</t>
+        </is>
+      </c>
+      <c r="G22" s="2" t="inlineStr">
+        <is>
+          <t>https://conf.theieie.org/2026s/</t>
+        </is>
+      </c>
+      <c r="H22" s="2" t="inlineStr"/>
+      <c r="I22" s="2" t="inlineStr"/>
+      <c r="J22" s="2" t="inlineStr"/>
+      <c r="K22" s="2" t="inlineStr"/>
+      <c r="L22" s="2" t="inlineStr"/>
+      <c r="M22" s="2" t="inlineStr"/>
+      <c r="N22" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="O22" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="P22" s="2" t="inlineStr">
+        <is>
+          <t>Conference</t>
+        </is>
+      </c>
+      <c r="Q22" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="R22" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="S22" s="2" t="n">
+        <v>130</v>
+      </c>
+      <c r="T22" s="2" t="inlineStr"/>
+      <c r="U22" s="2" t="inlineStr"/>
+      <c r="V22" s="2" t="inlineStr"/>
+      <c r="W22" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="X22" s="2" t="inlineStr">
+        <is>
+          <t>IMSI WEB_Publications</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>PUB_042</t>
+        </is>
+      </c>
+      <c r="B23" s="2" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C23" s="2" t="inlineStr">
+        <is>
+          <t>LEXIC: Lightweight Eye-tracking eXtension via Injected Complexity</t>
+        </is>
+      </c>
+      <c r="D23" s="2" t="inlineStr">
+        <is>
+          <t>IEEE Asia-Pacific Conf. on Circuits and Systems (APCCAS)</t>
+        </is>
+      </c>
+      <c r="E23" s="2" t="inlineStr">
+        <is>
+          <t>Sumin Lee, Kyeonghun Kim, Subeen Lee, Jiwon Yang, Tien Nguyen, Ken Ying-Kai Liao, Nam-Joon Kim†</t>
+        </is>
+      </c>
+      <c r="F23" s="2" t="inlineStr">
+        <is>
+          <t>https://arxiv.org/abs/2607.08152</t>
+        </is>
+      </c>
+      <c r="G23" s="2" t="inlineStr">
+        <is>
+          <t>https://apccas2026.org/</t>
+        </is>
+      </c>
+      <c r="H23" s="2" t="inlineStr"/>
+      <c r="I23" s="2" t="inlineStr"/>
+      <c r="J23" s="2" t="inlineStr"/>
+      <c r="K23" s="2" t="inlineStr"/>
+      <c r="L23" s="2" t="inlineStr"/>
+      <c r="M23" s="2" t="inlineStr">
+        <is>
+          <t>X(260704기준)</t>
+        </is>
+      </c>
+      <c r="N23" s="2" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="O23" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="P23" s="2" t="inlineStr">
+        <is>
+          <t>Conference</t>
+        </is>
+      </c>
+      <c r="Q23" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="R23" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="S23" s="2" t="n">
+        <v>140</v>
+      </c>
+      <c r="T23" s="2" t="inlineStr"/>
+      <c r="U23" s="2" t="inlineStr"/>
+      <c r="V23" s="2" t="inlineStr"/>
+      <c r="W23" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="X23" s="2" t="inlineStr">
+        <is>
+          <t>IMSI WEB_Publications</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>PUB_041</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C24" s="2" t="inlineStr">
+        <is>
+          <t>ProsMAE: Multi-Source MAE Pretraining for ISUP Grade Classification</t>
+        </is>
+      </c>
+      <c r="D24" s="2" t="inlineStr">
+        <is>
+          <t>IEEE Asia-Pacific Conf. on Circuits and Systems (APCCAS)</t>
+        </is>
+      </c>
+      <c r="E24" s="2" t="inlineStr">
+        <is>
+          <t>Anna Jung, Kyeonghun Kim, Youngung Han, Eunseob Choi, Jiwon Yang, Ken Ying-Kai Liao, Hyuk-Jae Lee, Nam-Joon Kim†</t>
+        </is>
+      </c>
+      <c r="F24" s="2" t="inlineStr">
+        <is>
+          <t>https://arxiv.org/abs/2607.08162</t>
+        </is>
+      </c>
+      <c r="G24" s="2" t="inlineStr">
+        <is>
+          <t>https://apccas2026.org/</t>
+        </is>
+      </c>
+      <c r="H24" s="2" t="inlineStr"/>
+      <c r="I24" s="2" t="inlineStr"/>
+      <c r="J24" s="2" t="inlineStr"/>
+      <c r="K24" s="2" t="inlineStr"/>
+      <c r="L24" s="2" t="inlineStr"/>
+      <c r="M24" s="2" t="inlineStr">
+        <is>
+          <t>X(260704기준)</t>
+        </is>
+      </c>
+      <c r="N24" s="2" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="O24" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="P24" s="2" t="inlineStr">
+        <is>
+          <t>Conference</t>
+        </is>
+      </c>
+      <c r="Q24" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="R24" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="S24" s="2" t="n">
+        <v>150</v>
+      </c>
+      <c r="T24" s="2" t="inlineStr"/>
+      <c r="U24" s="2" t="inlineStr"/>
+      <c r="V24" s="2" t="inlineStr"/>
+      <c r="W24" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="X24" s="2" t="inlineStr">
+        <is>
+          <t>IMSI WEB_Publications</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t>PUB_040</t>
+        </is>
+      </c>
+      <c r="B25" s="2" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C25" s="2" t="inlineStr">
+        <is>
+          <t>SCINTILLA-SNN: A Spiking Multi-Scale Selective Aggregation Network for Perineural Invasion Prediction</t>
+        </is>
+      </c>
+      <c r="D25" s="2" t="inlineStr">
+        <is>
+          <t>IEEE Asia-Pacific Conf. on Circuits and Systems (APCCAS)</t>
+        </is>
+      </c>
+      <c r="E25" s="2" t="inlineStr">
+        <is>
+          <t>Youngung Han, Yului Jung, Kyeonghun Kim, Dohyun Kweon, Suah Park, Hyunsu Go, Sungha Park, Anna Jung, Jinyong Jun, Woo Kyoung Jeong, Won Jae Lee, Ken Ying-Kai Liao, Hyuk-Jae Lee, Nam-Joon Kim†</t>
+        </is>
+      </c>
+      <c r="F25" s="2" t="inlineStr">
+        <is>
+          <t>https://drive.google.com/file/d/1WHeA_xlPgQxJhBD4B7JxEvdj7zJusy9s/view?usp=drive_link</t>
+        </is>
+      </c>
+      <c r="G25" s="2" t="inlineStr">
+        <is>
+          <t>https://apccas2026.org/</t>
+        </is>
+      </c>
+      <c r="H25" s="2" t="inlineStr"/>
+      <c r="I25" s="2" t="inlineStr"/>
+      <c r="J25" s="2" t="inlineStr"/>
+      <c r="K25" s="2" t="inlineStr"/>
+      <c r="L25" s="2" t="inlineStr"/>
+      <c r="M25" s="2" t="inlineStr">
+        <is>
+          <t>X(260704기준)</t>
+        </is>
+      </c>
+      <c r="N25" s="2" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="O25" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="P25" s="2" t="inlineStr">
+        <is>
+          <t>Conference</t>
+        </is>
+      </c>
+      <c r="Q25" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="R25" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="S25" s="2" t="n">
+        <v>160</v>
+      </c>
+      <c r="T25" s="2" t="inlineStr"/>
+      <c r="U25" s="2" t="inlineStr"/>
+      <c r="V25" s="2" t="inlineStr"/>
+      <c r="W25" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="X25" s="2" t="inlineStr">
+        <is>
+          <t>IMSI WEB_Publications</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>PUB_039</t>
+        </is>
+      </c>
+      <c r="B26" s="2" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C26" s="2" t="inlineStr">
+        <is>
+          <t>Order-Aware 2.5D Multiple Instance Learning for Preoperative MRI-Based Perineural Invasion Risk Assessment in Intrahepatic Cholangiocarcinoma</t>
+        </is>
+      </c>
+      <c r="D26" s="2" t="inlineStr">
+        <is>
+          <t>IEEE Asia-Pacific Conf. on Circuits and Systems (APCCAS)</t>
+        </is>
+      </c>
+      <c r="E26" s="2" t="inlineStr">
+        <is>
+          <t>Hyunsu Go, Youngung Han, Kyeonghun Kim, Jinyong Jun, Junbeom Lee, Dohyun Kweon, Yului Jung, Suah Park, Sungha Park, Anna Jung, Woo Kyoung Jeong, Ken Ying-Kai Liao, Hyuk-Jae Lee, Nam-Joon Kim†</t>
+        </is>
+      </c>
+      <c r="F26" s="2" t="inlineStr">
+        <is>
+          <t>https://drive.google.com/file/d/1uaJufvKOAzHjaxkXz84MWjmwVukz2hUP/view?usp=drive_link</t>
+        </is>
+      </c>
+      <c r="G26" s="2" t="inlineStr">
+        <is>
+          <t>https://apccas2026.org/</t>
+        </is>
+      </c>
+      <c r="H26" s="2" t="inlineStr"/>
+      <c r="I26" s="2" t="inlineStr"/>
+      <c r="J26" s="2" t="inlineStr"/>
+      <c r="K26" s="2" t="inlineStr"/>
+      <c r="L26" s="2" t="inlineStr"/>
+      <c r="M26" s="2" t="inlineStr"/>
+      <c r="N26" s="2" t="inlineStr"/>
+      <c r="O26" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="P26" s="2" t="inlineStr">
+        <is>
+          <t>Conference</t>
+        </is>
+      </c>
+      <c r="Q26" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="R26" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="S26" s="2" t="n">
+        <v>170</v>
+      </c>
+      <c r="T26" s="2" t="inlineStr"/>
+      <c r="U26" s="2" t="inlineStr"/>
+      <c r="V26" s="2" t="inlineStr"/>
+      <c r="W26" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="X26" s="2" t="inlineStr">
+        <is>
+          <t>IMSI WEB_Publications</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="inlineStr">
+        <is>
+          <t>PUB_038</t>
+        </is>
+      </c>
+      <c r="B27" s="2" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C27" s="2" t="inlineStr">
+        <is>
+          <t>Adaptive Routing and Local Context-Aware Token Selection in Diffusion Transformers for PNI Prediction</t>
+        </is>
+      </c>
+      <c r="D27" s="2" t="inlineStr">
+        <is>
+          <t>8th IEEE Int. Conf. on Artificial Intelligence Circuits and Systems (AICAS)</t>
+        </is>
+      </c>
+      <c r="E27" s="2" t="inlineStr">
+        <is>
+          <t>Youngung Han, Dohyun Kweon, Kyeonghun Kim, Hyunsu Go, Jina Jeong, Suah Park, Induk Um, Junga Kim, Anna Jung, Yului Jeong, Sungha Park, Jinyong Jun, Pa Hong, Woo Kyoung Jeong, Won Jae Lee, Ken Ying Kai Liao, Hyuk-Jae Lee, Nam-Joon Kim†</t>
+        </is>
+      </c>
+      <c r="F27" s="2" t="inlineStr">
+        <is>
+          <t>https://arxiv.org/abs/2607.11533</t>
+        </is>
+      </c>
+      <c r="G27" s="2" t="inlineStr">
+        <is>
+          <t>https://2026.ieee-aicas.org/</t>
+        </is>
+      </c>
+      <c r="H27" s="2" t="inlineStr"/>
+      <c r="I27" s="2" t="inlineStr"/>
+      <c r="J27" s="2" t="inlineStr"/>
+      <c r="K27" s="2" t="inlineStr"/>
+      <c r="L27" s="2" t="inlineStr"/>
+      <c r="M27" s="2" t="inlineStr">
+        <is>
+          <t>X(260704기준)</t>
+        </is>
+      </c>
+      <c r="N27" s="2" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="O27" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="P27" s="2" t="inlineStr">
+        <is>
+          <t>Conference</t>
+        </is>
+      </c>
+      <c r="Q27" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="R27" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="S27" s="2" t="n">
+        <v>180</v>
+      </c>
+      <c r="T27" s="2" t="inlineStr"/>
+      <c r="U27" s="2" t="inlineStr"/>
+      <c r="V27" s="2" t="inlineStr"/>
+      <c r="W27" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="X27" s="2" t="inlineStr">
+        <is>
+          <t>IMSI WEB_Publications</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="inlineStr">
+        <is>
+          <t>PUB_037</t>
+        </is>
+      </c>
+      <c r="B28" s="2" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C28" s="2" t="inlineStr">
+        <is>
+          <t>SpikeDS: Dual Sparsity Spikformer for Perineural Invasion Prediction in 3D MRI</t>
+        </is>
+      </c>
+      <c r="D28" s="2" t="inlineStr">
+        <is>
+          <t>8th IEEE Int. Conf. on Artificial Intelligence Circuits and Systems (AICAS)</t>
+        </is>
+      </c>
+      <c r="E28" s="2" t="inlineStr">
+        <is>
+          <t>Induk Um, Youngung Han, Kyeonghun Kim, Jina Jeong, Yului Jeong , Hyunsu Go,Dohyun Kweon, Anna Jung, Junga Kim, Sungha Park, Suah Park, Pa Hong, Woo Kyoung Jeong, Won Jae Lee, Ken Ying Kai Liao, Hyuk-Jae Lee, Nam-Joon Kim†</t>
+        </is>
+      </c>
+      <c r="F28" s="2" t="inlineStr">
+        <is>
+          <t>https://arxiv.org/abs/2607.11986</t>
+        </is>
+      </c>
+      <c r="G28" s="2" t="inlineStr">
+        <is>
+          <t>https://2026.ieee-aicas.org/</t>
+        </is>
+      </c>
+      <c r="H28" s="2" t="inlineStr"/>
+      <c r="I28" s="2" t="inlineStr"/>
+      <c r="J28" s="2" t="inlineStr"/>
+      <c r="K28" s="2" t="inlineStr"/>
+      <c r="L28" s="2" t="inlineStr"/>
+      <c r="M28" s="2" t="inlineStr">
+        <is>
+          <t>X(260704기준)</t>
+        </is>
+      </c>
+      <c r="N28" s="2" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="O28" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="P28" s="2" t="inlineStr">
+        <is>
+          <t>Conference</t>
+        </is>
+      </c>
+      <c r="Q28" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="R28" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="S28" s="2" t="n">
+        <v>190</v>
+      </c>
+      <c r="T28" s="2" t="inlineStr"/>
+      <c r="U28" s="2" t="inlineStr"/>
+      <c r="V28" s="2" t="inlineStr"/>
+      <c r="W28" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="X28" s="2" t="inlineStr">
+        <is>
+          <t>IMSI WEB_Publications</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="inlineStr">
+        <is>
+          <t>PUB_036</t>
+        </is>
+      </c>
+      <c r="B29" s="2" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C29" s="2" t="inlineStr">
+        <is>
+          <t>Anatomy-Privileged Distillation with Token Routing for MRI-Based Prediction of Perineural Invasion</t>
+        </is>
+      </c>
+      <c r="D29" s="2" t="inlineStr">
+        <is>
+          <t>8th IEEE Int. Conf. on Artificial Intelligence Circuits and Systems (AICAS)</t>
+        </is>
+      </c>
+      <c r="E29" s="2" t="inlineStr">
+        <is>
+          <t>Hyunsu Go, Youngung Han, Kyeonghun Kim, Junga Kim, Dohyun Kweon, Jinyong Jun, Sungha Park, Anna Jung, Induk Um, Yului Jeong, Suah Park, Jina Jeong, Suemin Yang, Pa Hong, Woo Kyoung Jeong, Won Jae Lee, Ken Ying Kai Liao, Hyuk-Jae Lee, Nam-Joon Kim†</t>
+        </is>
+      </c>
+      <c r="F29" s="2" t="inlineStr">
+        <is>
+          <t>https://arxiv.org/abs/2607.11987</t>
+        </is>
+      </c>
+      <c r="G29" s="2" t="inlineStr">
+        <is>
+          <t>https://2026.ieee-aicas.org/</t>
+        </is>
+      </c>
+      <c r="H29" s="2" t="inlineStr"/>
+      <c r="I29" s="2" t="inlineStr"/>
+      <c r="J29" s="2" t="inlineStr"/>
+      <c r="K29" s="2" t="inlineStr"/>
+      <c r="L29" s="2" t="inlineStr"/>
+      <c r="M29" s="2" t="inlineStr">
+        <is>
+          <t>X(260704기준)</t>
+        </is>
+      </c>
+      <c r="N29" s="2" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="O29" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="P29" s="2" t="inlineStr">
+        <is>
+          <t>Conference</t>
+        </is>
+      </c>
+      <c r="Q29" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="R29" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="S29" s="2" t="n">
+        <v>200</v>
+      </c>
+      <c r="T29" s="2" t="inlineStr"/>
+      <c r="U29" s="2" t="inlineStr"/>
+      <c r="V29" s="2" t="inlineStr"/>
+      <c r="W29" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="X29" s="2" t="inlineStr">
+        <is>
+          <t>IMSI WEB_Publications</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="inlineStr">
+        <is>
+          <t>PUB_035</t>
+        </is>
+      </c>
+      <c r="B30" s="2" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C30" s="2" t="inlineStr">
+        <is>
+          <t>3D-LLDM: LABEL-GUIDED 3D LATENT DIFFUSION MODEL FOR IMPROVING HIGH-RESOLUTION SYNTHETIC MR IMAGING IN HEPATIC STRUCTURE SEGMENTATION</t>
+        </is>
+      </c>
+      <c r="D30" s="2" t="inlineStr">
+        <is>
+          <t>2026 IEEE 23rd International Symposium on Biomedical Imaging (ISBI 2026), Oral Presentation</t>
+        </is>
+      </c>
+      <c r="E30" s="2" t="inlineStr">
+        <is>
+          <t>Kyeonghun Kim, Jaehyeok Bae, Youngung Han, Joo Young Bae, Seoyoung Ju, Junsu Lim, Gyeongmin Kim, Woo Kyoung Jeong, Ken Ying-Kai Liao, Won Jae Lee, Pa Hong, Hyuk-Jae Lee, Nam-Joon Kim†</t>
+        </is>
+      </c>
+      <c r="F30" s="2" t="inlineStr">
+        <is>
+          <t>https://arxiv.org/abs/2603.23845</t>
+        </is>
+      </c>
+      <c r="G30" s="2" t="inlineStr">
+        <is>
+          <t>https://biomedicalimaging.org/2026/</t>
+        </is>
+      </c>
+      <c r="H30" s="2" t="inlineStr"/>
+      <c r="I30" s="2" t="inlineStr">
+        <is>
+          <t>https://github.com/khkim1729/3D-LLDM</t>
+        </is>
+      </c>
+      <c r="J30" s="2" t="inlineStr">
+        <is>
+          <t>https://drive.google.com/file/d/1mftbV7-XWdl3k3FDau8Vv8MZddhJ8oGK/view?usp=sharing</t>
+        </is>
+      </c>
+      <c r="K30" s="2" t="inlineStr">
+        <is>
+          <t>https://drive.google.com/file/d/1HiPJ39iSo-M0jlet5I_0KT5dAdbokalh/view?usp=drive_link</t>
+        </is>
+      </c>
+      <c r="L30" s="2" t="inlineStr">
+        <is>
+          <t>@inproceedings{kim20263d,
+  title={3D-LLDM: Label-Guided 3D Latent Diffusion Model for Improving High-Resolution Synthetic MR Imaging in Hepatic Structure Segmentation},
+  author={Kim, Kyeonghun and Bae, Jaehyeok and Han, Youngung and Bae, Joo Young and Ju, Seoyoung and Lim, Junsu and Kim, Gyeongmin and Kim, Nam-Joon and Jeong, Woo Kyoung and Liao, Ken Ying-Kai and others},
+  booktitle={2026 IEEE 23rd International Symposium on Biomedical Imaging (ISBI)},
+  pages={1–––––––––––––––––––––––––––––––5},
+  year={2026},
+  organization={IEEE}
+}</t>
+        </is>
+      </c>
+      <c r="M30" s="2" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="N30" s="2" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="O30" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="P30" s="2" t="inlineStr">
+        <is>
+          <t>Conference</t>
+        </is>
+      </c>
+      <c r="Q30" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="R30" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="S30" s="2" t="n">
+        <v>210</v>
+      </c>
+      <c r="T30" s="2" t="inlineStr"/>
+      <c r="U30" s="2" t="inlineStr"/>
+      <c r="V30" s="2" t="inlineStr"/>
+      <c r="W30" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="X30" s="2" t="inlineStr">
+        <is>
+          <t>IMSI WEB_Publications</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="2" t="inlineStr">
+        <is>
+          <t>PUB_034</t>
+        </is>
+      </c>
+      <c r="B31" s="2" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C31" s="2" t="inlineStr">
+        <is>
+          <t>MMA-Former: Multi-Window Mixture-of-Head Attention Transformer for Adaptive PNI Prediction in 3D MRI</t>
+        </is>
+      </c>
+      <c r="D31" s="2" t="inlineStr">
+        <is>
+          <t>2026 IEEE 23rd International Symposium on Biomedical Imaging (ISBI 2026), Oral Presentation</t>
+        </is>
+      </c>
+      <c r="E31" s="2" t="inlineStr">
+        <is>
+          <t>Youngung Han, Induk Um, Kyeonghun Kim, Junga Kim, Hyunsu Go, Jaewon Jung, Woo Kyoung Jeong†, Won Jae Lee, Ken Ying-Kai Liao, Pa Hong, Hyuk-Jae Lee, Nam-Joon Kim†</t>
+        </is>
+      </c>
+      <c r="F31" s="2" t="inlineStr">
+        <is>
+          <t>https://arxiv.org/abs/2607.10988</t>
+        </is>
+      </c>
+      <c r="G31" s="2" t="inlineStr">
+        <is>
+          <t>https://biomedicalimaging.org/2026/</t>
+        </is>
+      </c>
+      <c r="H31" s="2" t="inlineStr"/>
+      <c r="I31" s="2" t="inlineStr">
+        <is>
+          <t>https://github.com/khkim1729/MAEgic</t>
+        </is>
+      </c>
+      <c r="J31" s="2" t="inlineStr">
+        <is>
+          <t>https://drive.google.com/file/d/12Hc7rvhjkuc640BqzIbnKFGVCoInGj44/view?usp=sharing</t>
+        </is>
+      </c>
+      <c r="K31" s="2" t="inlineStr">
+        <is>
+          <t>https://drive.google.com/file/d/1hn1x2v-DlYPvobwQh2au2swaB_bOLZgA/view?usp=drive_link</t>
+        </is>
+      </c>
+      <c r="L31" s="2" t="inlineStr">
+        <is>
+          <t>@inproceedings{han2026mma,
+  title={MMA-Former: Multi-Window Mixture-of-Head Attention Transformer for Adaptive PNI Prediction in 3D MRI},
+  author={Han, Youngung and Um, Induk and Kim, Kyeonghun and Kim, Junga and Go, Hyunsu and Jung, Jaewon and Kim, Nam-Joon and Jeong, Woo Kyoung and Lee, Won Jae and Hong, Pa and others},
+  booktitle={2026 IEEE 23rd International Symposium on Biomedical Imaging (ISBI)},
+  pages={1–5},
+  year={2026},
+  organization={IEEE}
+}</t>
+        </is>
+      </c>
+      <c r="M31" s="2" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="N31" s="2" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="O31" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="P31" s="2" t="inlineStr">
+        <is>
+          <t>Conference</t>
+        </is>
+      </c>
+      <c r="Q31" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="R31" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="S31" s="2" t="n">
+        <v>220</v>
+      </c>
+      <c r="T31" s="2" t="inlineStr"/>
+      <c r="U31" s="2" t="inlineStr"/>
+      <c r="V31" s="2" t="inlineStr"/>
+      <c r="W31" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="X31" s="2" t="inlineStr">
+        <is>
+          <t>IMSI WEB_Publications</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="2" t="inlineStr">
+        <is>
+          <t>PUB_033</t>
+        </is>
+      </c>
+      <c r="B32" s="2" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C32" s="2" t="inlineStr">
+        <is>
+          <t>LoSA-Net: A Localized and Scale-Adaptive Network for Boundary-Sensitive Prediction of Perineural Invasion in 3D MRI</t>
+        </is>
+      </c>
+      <c r="D32" s="2" t="inlineStr">
+        <is>
+          <t>2026 IEEE 23rd International Symposium on Biomedical Imaging (ISBI 2026), Oral Presentation</t>
+        </is>
+      </c>
+      <c r="E32" s="2" t="inlineStr">
+        <is>
+          <t>Youngung Han, Hyunsu Go, Kyeonghun Kim, Induk Um, Junga Kim, Jaewon Jung, Woo Kyoung Jeong†, Won Jae Lee, Ken Ying-Kai Liao, Pa Hong, Hyuk-Jae Lee, Nam-Joon Kim†</t>
+        </is>
+      </c>
+      <c r="F32" s="2" t="inlineStr">
+        <is>
+          <t>https://arxiv.org/abs/2607.10992</t>
+        </is>
+      </c>
+      <c r="G32" s="2" t="inlineStr">
+        <is>
+          <t>https://biomedicalimaging.org/2026/</t>
+        </is>
+      </c>
+      <c r="H32" s="2" t="inlineStr"/>
+      <c r="I32" s="2" t="inlineStr">
+        <is>
+          <t>https://github.com/khkim1729/COTTUS</t>
+        </is>
+      </c>
+      <c r="J32" s="2" t="inlineStr">
+        <is>
+          <t>https://drive.google.com/file/d/1OWqMKs0wLtwm9DEdIDqof93lPMtqfDaQ/view?usp=sharing</t>
+        </is>
+      </c>
+      <c r="K32" s="2" t="inlineStr">
+        <is>
+          <t>https://drive.google.com/file/d/12-bLxqc-Mwzt9GYcI75N9ecftrkPU-ym/view?usp=drive_link</t>
+        </is>
+      </c>
+      <c r="L32" s="2" t="inlineStr">
+        <is>
+          <t>@inproceedings{han2026losa,
+  title={Losa-Net: A Localized and Scale-Adaptive Network for Boundary-Sensitive Prediction of Perineural Invasion in 3D MRI},
+  author={Han, Youngung and Go, Hyunsu and Kim, Kyeonghun and Um, Induk and Kim, Junga and Jung, Jaewon and Kim, Nam-Joon and Jeong, Woo Kyoung and Lee, Won Jae and Liao, Ken Ying-Kai and others},
+  booktitle={2026 IEEE 23rd International Symposium on Biomedical Imaging (ISBI)},
+  pages={1–––––––––––––––––––––––––––––––5},
+  year={2026},
+  organization={IEEE}
+}</t>
+        </is>
+      </c>
+      <c r="M32" s="2" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="N32" s="2" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="O32" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="P32" s="2" t="inlineStr">
+        <is>
+          <t>Conference</t>
+        </is>
+      </c>
+      <c r="Q32" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="R32" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="S32" s="2" t="n">
+        <v>230</v>
+      </c>
+      <c r="T32" s="2" t="inlineStr"/>
+      <c r="U32" s="2" t="inlineStr"/>
+      <c r="V32" s="2" t="inlineStr"/>
+      <c r="W32" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="X32" s="2" t="inlineStr">
+        <is>
+          <t>IMSI WEB_Publications</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="2" t="inlineStr">
+        <is>
+          <t>PUB_032</t>
+        </is>
+      </c>
+      <c r="B33" s="2" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C33" s="2" t="inlineStr">
+        <is>
+          <t>GRAVEX: GPU-accelerated GAN-Diffusion Representation for counterfeit pattern Analysis with MONAI-based Validation &amp; Examination</t>
+        </is>
+      </c>
+      <c r="D33" s="2" t="inlineStr">
+        <is>
+          <t>NVIDIA GTC 2026</t>
+        </is>
+      </c>
+      <c r="E33" s="2" t="inlineStr">
+        <is>
+          <t>Kyeonghun Kim, Eunseob Choi, Junsu Lim, Induk Um, Ken Ying-Kai Liao, Hyuk-jae Lee</t>
+        </is>
+      </c>
+      <c r="F33" s="2" t="inlineStr">
+        <is>
+          <t>https://drive.google.com/file/d/1g2Gz-rDwRo56fjrXWHTcutVtWx6VVTGl/view?usp=drive_link</t>
+        </is>
+      </c>
+      <c r="G33" s="2" t="inlineStr">
+        <is>
+          <t>https://www.nvidia.com/gtc/session-catalog/sessions/gtc26-p81285/</t>
+        </is>
+      </c>
+      <c r="H33" s="2" t="inlineStr"/>
+      <c r="I33" s="2" t="inlineStr"/>
+      <c r="J33" s="2" t="inlineStr"/>
+      <c r="K33" s="2" t="inlineStr"/>
+      <c r="L33" s="2" t="inlineStr"/>
+      <c r="M33" s="2" t="inlineStr"/>
+      <c r="N33" s="2" t="inlineStr"/>
+      <c r="O33" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="P33" s="2" t="inlineStr">
+        <is>
+          <t>Conference</t>
+        </is>
+      </c>
+      <c r="Q33" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="R33" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="S33" s="2" t="n">
+        <v>240</v>
+      </c>
+      <c r="T33" s="2" t="inlineStr"/>
+      <c r="U33" s="2" t="inlineStr"/>
+      <c r="V33" s="2" t="inlineStr"/>
+      <c r="W33" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="X33" s="2" t="inlineStr">
+        <is>
+          <t>IMSI WEB_Publications</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="2" t="inlineStr">
+        <is>
+          <t>PUB_031</t>
+        </is>
+      </c>
+      <c r="B34" s="2" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C34" s="2" t="inlineStr">
+        <is>
+          <t>RAPIDS: Real-time Accelerated Pipeline for Intelligent Dental Segmentation</t>
+        </is>
+      </c>
+      <c r="D34" s="2" t="inlineStr">
+        <is>
+          <t>NVIDIA GTC 2026</t>
+        </is>
+      </c>
+      <c r="E34" s="2" t="inlineStr">
+        <is>
+          <t>Kyeonghun Kim, Youngung Han, Hyeonseok Jung, Gyeongmin Kim, Ken Ying-Kai Liao, Nam-Joon Kim†</t>
+        </is>
+      </c>
+      <c r="F34" s="2" t="inlineStr">
+        <is>
+          <t>https://drive.google.com/file/d/13G5yTcfwH9vDGJPxSJXbvXf-Su_UMM1E/view?usp=drive_link</t>
+        </is>
+      </c>
+      <c r="G34" s="2" t="inlineStr">
+        <is>
+          <t>https://www.nvidia.com/gtc/session-catalog/sessions/gtc26-p81266/</t>
+        </is>
+      </c>
+      <c r="H34" s="2" t="inlineStr"/>
+      <c r="I34" s="2" t="inlineStr"/>
+      <c r="J34" s="2" t="inlineStr"/>
+      <c r="K34" s="2" t="inlineStr"/>
+      <c r="L34" s="2" t="inlineStr"/>
+      <c r="M34" s="2" t="inlineStr"/>
+      <c r="N34" s="2" t="inlineStr"/>
+      <c r="O34" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="P34" s="2" t="inlineStr">
+        <is>
+          <t>Conference</t>
+        </is>
+      </c>
+      <c r="Q34" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="R34" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="S34" s="2" t="n">
+        <v>250</v>
+      </c>
+      <c r="T34" s="2" t="inlineStr"/>
+      <c r="U34" s="2" t="inlineStr"/>
+      <c r="V34" s="2" t="inlineStr"/>
+      <c r="W34" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="X34" s="2" t="inlineStr">
+        <is>
+          <t>IMSI WEB_Publications</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="2" t="inlineStr">
+        <is>
+          <t>PUB_029</t>
+        </is>
+      </c>
+      <c r="B35" s="2" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C35" s="2" t="inlineStr">
+        <is>
+          <t>NeoNet: Neoplastic End-to-End Original 3D MRI-Based Deep Learning Framework for Prediction of Perineural Invasion: From Segmentation to Generation-driven Classification</t>
+        </is>
+      </c>
+      <c r="D35" s="2" t="inlineStr">
+        <is>
+          <t>Workshop on Health Intelligence (W3PHIAI), AAAI26 Oral Presentation</t>
+        </is>
+      </c>
+      <c r="E35" s="2" t="inlineStr">
+        <is>
+          <t>Youngung Han, Minkyung Cha, Kyeonghun Kim, Induk Um, Myeongbin So, Joo Young Bae, Jaewon Jung, Jung Hyeok Park, Woo Kyoung Jeong*, Won Jae Lee, Pa Hong, Ken Ying-Kai Liao, Hyuk-Jae Lee, Nam-Joon Kim†</t>
+        </is>
+      </c>
+      <c r="F35" s="2" t="inlineStr">
+        <is>
+          <t>https://arxiv.org/pdf/2603.29449</t>
+        </is>
+      </c>
+      <c r="G35" s="2" t="inlineStr">
+        <is>
+          <t>https://w3phiai2026.w3phi.com/index.html</t>
+        </is>
+      </c>
+      <c r="H35" s="2" t="inlineStr"/>
+      <c r="I35" s="2" t="inlineStr"/>
+      <c r="J35" s="2" t="inlineStr"/>
+      <c r="K35" s="2" t="inlineStr">
+        <is>
+          <t>https://drive.google.com/file/d/13zeMYsYSVunVH5N1S3Ln3zPLQrUzcqQa/view</t>
+        </is>
+      </c>
+      <c r="L35" s="2" t="inlineStr">
+        <is>
+          <t>@article{han2026neonet,
+  title={NeoNet: An End-to-End 3D MRI-Based Deep Learning Framework for Non-Invasive Prediction of Perineural Invasion via Generation-Driven Classification},
+  author={Han, Youngung and Cha, Minkyung and Kim, Kyeonghun and Um, Induk and Sho, Myeongbin and Bae, Joo Young and Jung, Jaewon and Park, Jung Hyeok and Lee, Seojun and Kim, Nam-Joon and others},
+  journal={arXiv preprint arXiv:2603.29449},
+  year={2026}
+}</t>
+        </is>
+      </c>
+      <c r="M35" s="2" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="N35" s="2" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="O35" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="P35" s="2" t="inlineStr">
+        <is>
+          <t>Conference</t>
+        </is>
+      </c>
+      <c r="Q35" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="R35" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="S35" s="2" t="n">
+        <v>270</v>
+      </c>
+      <c r="T35" s="2" t="inlineStr"/>
+      <c r="U35" s="2" t="inlineStr"/>
+      <c r="V35" s="2" t="inlineStr"/>
+      <c r="W35" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="X35" s="2" t="inlineStr">
+        <is>
+          <t>IMSI WEB_Publications</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="2" t="inlineStr">
+        <is>
+          <t>PUB_028</t>
+        </is>
+      </c>
+      <c r="B36" s="2" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C36" s="2" t="inlineStr">
+        <is>
+          <t>COTTA: Context-Aware Transfer Adaptation for Trajectory Prediction in Autonomous Driving</t>
+        </is>
+      </c>
+      <c r="D36" s="2" t="inlineStr">
+        <is>
+          <t>IEEE Int. Conf. Electronics, Information, and Communication (ICEIC)</t>
+        </is>
+      </c>
+      <c r="E36" s="2" t="inlineStr">
+        <is>
+          <t>Seohyeong Park, Jaeyeol Lim, Seoyoung Ju, Kyeonghun Kim, Ken Ying-Kai Liao, Hyuk-Jae Lee, Nam-Joon Kim†</t>
+        </is>
+      </c>
+      <c r="F36" s="2" t="inlineStr">
+        <is>
+          <t>https://arxiv.org/abs/2604.00402</t>
+        </is>
+      </c>
+      <c r="G36" s="2" t="inlineStr">
+        <is>
+          <t>https://iceic.org/2026/</t>
+        </is>
+      </c>
+      <c r="H36" s="2" t="inlineStr"/>
+      <c r="I36" s="2" t="inlineStr">
+        <is>
+          <t>https://github.com/khkim1729/COTTUS</t>
+        </is>
+      </c>
+      <c r="J36" s="2" t="inlineStr">
+        <is>
+          <t>https://drive.google.com/file/d/1OWqMKs0wLtwm9DEdIDqof93lPMtqfDaQ/view?usp=sharing</t>
+        </is>
+      </c>
+      <c r="K36" s="2" t="inlineStr">
+        <is>
+          <t>https://drive.google.com/file/d/1haddFfwmRb3lFlNVbTGn8_GuqbhntSNP/view?usp=drive_link</t>
+        </is>
+      </c>
+      <c r="L36" s="2" t="inlineStr"/>
+      <c r="M36" s="2" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="N36" s="2" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="O36" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="P36" s="2" t="inlineStr">
+        <is>
+          <t>Conference</t>
+        </is>
+      </c>
+      <c r="Q36" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="R36" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="S36" s="2" t="n">
+        <v>280</v>
+      </c>
+      <c r="T36" s="2" t="inlineStr"/>
+      <c r="U36" s="2" t="inlineStr"/>
+      <c r="V36" s="2" t="inlineStr"/>
+      <c r="W36" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="X36" s="2" t="inlineStr">
+        <is>
+          <t>IMSI WEB_Publications</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="2" t="inlineStr">
+        <is>
+          <t>PUB_027</t>
+        </is>
+      </c>
+      <c r="B37" s="2" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C37" s="2" t="inlineStr">
+        <is>
+          <t>MAESIL: Masked Autoencoder for Enhanced Self-supervised Medical Image Learning</t>
+        </is>
+      </c>
+      <c r="D37" s="2" t="inlineStr">
+        <is>
+          <t>IEEE Int. Conf. Electronics, Information, and Communication (ICEIC)</t>
+        </is>
+      </c>
+      <c r="E37" s="2" t="inlineStr">
+        <is>
+          <t>Kyeonghun Kim, Hyeonseok Jung, Youngung Han, Seongbin Park, Eunseob Choi, Hyunsu Go, Seoyoung Ju, Seohyeong Park, Gyeongmin Kim, MinJu Kwon, KyungSeok Yuh, Soo Yong Kim, Ken Ying-Kai Liao, Hyuk-Jae Lee, Nam-Joon Kim†</t>
+        </is>
+      </c>
+      <c r="F37" s="2" t="inlineStr">
+        <is>
+          <t>https://arxiv.org/abs/2604.00514</t>
+        </is>
+      </c>
+      <c r="G37" s="2" t="inlineStr">
+        <is>
+          <t>https://iceic.org/2026/</t>
+        </is>
+      </c>
+      <c r="H37" s="2" t="inlineStr"/>
+      <c r="I37" s="2" t="inlineStr">
+        <is>
+          <t>https://github.com/khkim1729/MAEgic</t>
+        </is>
+      </c>
+      <c r="J37" s="2" t="inlineStr">
+        <is>
+          <t>https://drive.google.com/file/d/12Hc7rvhjkuc640BqzIbnKFGVCoInGj44/view?usp=sharing</t>
+        </is>
+      </c>
+      <c r="K37" s="2" t="inlineStr">
+        <is>
+          <t>https://drive.google.com/file/d/1haddFfwmRb3lFlNVbTGn8_GuqbhntSNP/view?usp=drive_link</t>
+        </is>
+      </c>
+      <c r="L37" s="2" t="inlineStr">
+        <is>
+          <t>@inproceedings{kim2026maesil,
+  title={MAESIL: Masked Autoencoder for Enhanced Self-supervised Medical Image Learning},
+  author={Kim, Kyeonghun and Jung, Hyeonseok and Han, Youngung and Lim, Junsu and Jean, Yeonju and Park, Seongbin and Choi, Eunseob and Go, Hyunsu and Ju, Seoyoung and Park, Seohyoung and others},
+  booktitle={2026 International Conference on Electronics, Information, and Communication (ICEIC)},
+  pages={1–––––––––––––––––––––––––––––––5},
+  year={2026},
+  organization={IEEE}
+}</t>
+        </is>
+      </c>
+      <c r="M37" s="2" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="N37" s="2" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="O37" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="P37" s="2" t="inlineStr">
+        <is>
+          <t>Conference</t>
+        </is>
+      </c>
+      <c r="Q37" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="R37" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="S37" s="2" t="n">
+        <v>290</v>
+      </c>
+      <c r="T37" s="2" t="inlineStr"/>
+      <c r="U37" s="2" t="inlineStr"/>
+      <c r="V37" s="2" t="inlineStr"/>
+      <c r="W37" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="X37" s="2" t="inlineStr">
+        <is>
+          <t>IMSI WEB_Publications</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="2" t="inlineStr">
+        <is>
+          <t>PUB_025</t>
+        </is>
+      </c>
+      <c r="B38" s="2" t="n">
+        <v>2025</v>
+      </c>
+      <c r="C38" s="2" t="inlineStr">
+        <is>
+          <t>Improving Deep Learning-based Diagnosis of Hepatic Tumors on Multi-phase Contrast-enhanced Ultrasound Images: Comparison of Padding Strategies</t>
+        </is>
+      </c>
+      <c r="D38" s="2" t="inlineStr">
+        <is>
+          <t>ULTRASONICS</t>
+        </is>
+      </c>
+      <c r="E38" s="2" t="inlineStr">
+        <is>
+          <t>Taehoon Lee, Jaeyeol Lim, Woo Kyoung Jeong, Won Jae Lee, Kyeonghun Kim, Nam-Joon Kim†</t>
+        </is>
+      </c>
+      <c r="F38" s="2" t="inlineStr">
+        <is>
+          <t>https://drive.google.com/file/d/1iyHjwofS3oMK8-FA3a3_1LYQYClR_6Nu/view?usp=drive_link</t>
+        </is>
+      </c>
+      <c r="G38" s="2" t="inlineStr"/>
+      <c r="H38" s="2" t="inlineStr"/>
+      <c r="I38" s="2" t="inlineStr">
+        <is>
+          <t>https://github.com/khkim1729/LUCAS</t>
+        </is>
+      </c>
+      <c r="J38" s="2" t="inlineStr">
+        <is>
+          <t>https://drive.google.com/file/d/1U3u5KY8L8bolu2r9Cd4uKXiYOPxCdPxo/view?usp=drive_link</t>
+        </is>
+      </c>
+      <c r="K38" s="2" t="inlineStr"/>
+      <c r="L38" s="2" t="inlineStr"/>
+      <c r="M38" s="2" t="inlineStr"/>
+      <c r="N38" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="O38" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="P38" s="2" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="Q38" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="R38" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="S38" s="2" t="n">
+        <v>310</v>
+      </c>
+      <c r="T38" s="2" t="inlineStr"/>
+      <c r="U38" s="2" t="inlineStr"/>
+      <c r="V38" s="2" t="inlineStr"/>
+      <c r="W38" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="X38" s="2" t="inlineStr">
+        <is>
+          <t>IMSI WEB_Publications</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="2" t="inlineStr">
+        <is>
+          <t>PUB_024</t>
+        </is>
+      </c>
+      <c r="B39" s="2" t="n">
+        <v>2025</v>
+      </c>
+      <c r="C39" s="2" t="inlineStr">
+        <is>
+          <t>CIPHER: Counterfeit Image Pattern High-level Examination via Representation for GAN and Diffusion Discriminator Learning</t>
+        </is>
+      </c>
+      <c r="D39" s="2" t="inlineStr">
+        <is>
+          <t>IEEE ICCE-Asia</t>
+        </is>
+      </c>
+      <c r="E39" s="2" t="inlineStr">
+        <is>
+          <t>Kyeonghun Kim, Youngung Han, Seoyoung Ju, Yeonju Jeon, YooHyun Kim, Minseo Choi, SuYeon Lim, Kyungtae Park, Seungwoo Baek, Sieun Hyeon*, Hyuk-Jae Lee, Nam-Joon Kim†</t>
+        </is>
+      </c>
+      <c r="F39" s="2" t="inlineStr">
+        <is>
+          <t>https://arxiv.org/abs/2603.29356</t>
+        </is>
+      </c>
+      <c r="G39" s="2" t="inlineStr">
+        <is>
+          <t>https://icce-asia2025.org/2025/</t>
+        </is>
+      </c>
+      <c r="H39" s="2" t="inlineStr"/>
+      <c r="I39" s="2" t="inlineStr">
+        <is>
+          <t>https://github.com/outta-ai/2025_OUTTA_AIBootcamp_Deep-Learning_final_project</t>
+        </is>
+      </c>
+      <c r="J39" s="2" t="inlineStr">
+        <is>
+          <t>https://drive.google.com/file/d/1U3u5KY8L8bolu2r9Cd4uKXiYOPxCdPxo/view</t>
+        </is>
+      </c>
+      <c r="K39" s="2" t="inlineStr"/>
+      <c r="L39" s="2" t="inlineStr">
+        <is>
+          <t>@article{kim2026cipher,
+  title={CIPHER: Counterfeit Image Pattern High-level Examination via Representation},
+  author={Kim, Kyeonghun and Han, Youngung and Ju, Seoyoung and Jean, Yeonju and Kim, YooHyun and Choi, Minseo and Lim, SuYeon and Park, Kyungtae and Baek, Seungwoo and Hyeon, Sieun and others},
+  journal={arXiv preprint arXiv:2603.29356},
+  year={2026}
+}</t>
+        </is>
+      </c>
+      <c r="M39" s="2" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="N39" s="2" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="O39" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="P39" s="2" t="inlineStr">
+        <is>
+          <t>Conference</t>
+        </is>
+      </c>
+      <c r="Q39" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="R39" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="S39" s="2" t="n">
+        <v>320</v>
+      </c>
+      <c r="T39" s="2" t="inlineStr"/>
+      <c r="U39" s="2" t="inlineStr"/>
+      <c r="V39" s="2" t="inlineStr"/>
+      <c r="W39" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="X39" s="2" t="inlineStr">
+        <is>
+          <t>IMSI WEB_Publications</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="2" t="inlineStr">
+        <is>
+          <t>PUB_023</t>
+        </is>
+      </c>
+      <c r="B40" s="2" t="n">
+        <v>2025</v>
+      </c>
+      <c r="C40" s="2" t="inlineStr">
+        <is>
+          <t>Feasibility Study of QCNet for Korean Road Adaptation and Optimal Training Strategies</t>
+        </is>
+      </c>
+      <c r="D40" s="2" t="inlineStr">
+        <is>
+          <t>IEIE 2025 Autumn (대한전자공학회 추계학술대회)</t>
+        </is>
+      </c>
+      <c r="E40" s="2" t="inlineStr">
+        <is>
+          <t>Seohyeong Park, Jaeyeol Iim, Seoyoung Ju, Kyeonghun Kim, Nam-joon Kim†, Hyuk-Jae Lee, Nam-Joon Kim†</t>
+        </is>
+      </c>
+      <c r="F40" s="2" t="inlineStr">
+        <is>
+          <t>https://drive.google.com/file/d/1I2cqKpUNs4CtjnXXaEviFagiQr0_EMlo/view?usp=sharing</t>
+        </is>
+      </c>
+      <c r="G40" s="2" t="inlineStr"/>
+      <c r="H40" s="2" t="inlineStr"/>
+      <c r="I40" s="2" t="inlineStr"/>
+      <c r="J40" s="2" t="inlineStr">
+        <is>
+          <t>https://drive.google.com/file/d/1u6t5V5BqKTnKABlbThzg9er5ulXgV3PH/view?usp=sharing</t>
+        </is>
+      </c>
+      <c r="K40" s="2" t="inlineStr"/>
+      <c r="L40" s="2" t="inlineStr"/>
+      <c r="M40" s="2" t="inlineStr"/>
+      <c r="N40" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="O40" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="P40" s="2" t="inlineStr">
+        <is>
+          <t>Conference</t>
+        </is>
+      </c>
+      <c r="Q40" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="R40" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="S40" s="2" t="n">
+        <v>330</v>
+      </c>
+      <c r="T40" s="2" t="inlineStr"/>
+      <c r="U40" s="2" t="inlineStr"/>
+      <c r="V40" s="2" t="inlineStr"/>
+      <c r="W40" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="X40" s="2" t="inlineStr">
+        <is>
+          <t>IMSI WEB_Publications</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="2" t="inlineStr">
+        <is>
+          <t>PUB_021</t>
+        </is>
+      </c>
+      <c r="B41" s="2" t="n">
+        <v>2025</v>
+      </c>
+      <c r="C41" s="2" t="inlineStr">
+        <is>
+          <t>ControlNet-Guided Latent Diffusion for Tumor-Conditioned 3D Liver MRI Generation</t>
+        </is>
+      </c>
+      <c r="D41" s="2" t="inlineStr">
+        <is>
+          <t>IEIE 2025 Summer (대한전자공학회 하계학술대회)</t>
+        </is>
+      </c>
+      <c r="E41" s="2" t="inlineStr">
+        <is>
+          <t>Minkyung Cha, Kyeonghun Kim, Youngung Han, Joo Young Bae, Seoyoung Ju, Induk Um, Chaeyoung Lee, Myeongbin So, Suyeon Lim, Yeonju Jeon, Minju Kwon, Hyeonseok Jung, Kyeongseok Yu, Seohyeong Park, Sunghoon Park, Soo Yong Kim, Yoonkyoung Chun, Minjae Park, Seonghun Park, Pa Hong, Won Jae Lee, Woo Kyoung Jeong, Jihye Min, Hyuk-Jae Lee, Nam-Joon Kim†</t>
+        </is>
+      </c>
+      <c r="F41" s="2" t="inlineStr">
+        <is>
+          <t>https://drive.google.com/file/d/1AyrPobIThqZ4CdTTd05f8FFz2gA7blkB/view?usp=sharing</t>
+        </is>
+      </c>
+      <c r="G41" s="2" t="inlineStr"/>
+      <c r="H41" s="2" t="inlineStr"/>
+      <c r="I41" s="2" t="inlineStr"/>
+      <c r="J41" s="2" t="inlineStr"/>
+      <c r="K41" s="2" t="inlineStr"/>
+      <c r="L41" s="2" t="inlineStr"/>
+      <c r="M41" s="2" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="N41" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="O41" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="P41" s="2" t="inlineStr">
+        <is>
+          <t>Conference</t>
+        </is>
+      </c>
+      <c r="Q41" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="R41" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="S41" s="2" t="n">
+        <v>350</v>
+      </c>
+      <c r="T41" s="2" t="inlineStr"/>
+      <c r="U41" s="2" t="inlineStr"/>
+      <c r="V41" s="2" t="inlineStr"/>
+      <c r="W41" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="X41" s="2" t="inlineStr">
+        <is>
+          <t>IMSI WEB_Publications</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="2" t="inlineStr">
+        <is>
+          <t>PUB_020</t>
+        </is>
+      </c>
+      <c r="B42" s="2" t="n">
+        <v>2025</v>
+      </c>
+      <c r="C42" s="2" t="inlineStr">
+        <is>
+          <t>FOSCU: Feasibility of Synthetic MRI Generation via Duo-Diffusion Models for Enhancement of 3D U-Nets in Hepatic Segmentation</t>
+        </is>
+      </c>
+      <c r="D42" s="2" t="inlineStr">
+        <is>
+          <t>IEEE Asia-Pacific Conf. on Circuits and Systems (APCCAS)</t>
+        </is>
+      </c>
+      <c r="E42" s="2" t="inlineStr">
+        <is>
+          <t>Youngung Han*, Kyeonghun Kim, Seoyoung Ju, Yeonju Jeon, Minkyung Cha, Seohyeong Park, Hyeonseok Jung, Woo Kyoung Jeong, Ken Ying-Kai Liao, Hyuk-Jae Lee, Nam-Joon Kim†</t>
+        </is>
+      </c>
+      <c r="F42" s="2" t="inlineStr">
+        <is>
+          <t>https://arxiv.org/abs/2603.29343</t>
+        </is>
+      </c>
+      <c r="G42" s="2" t="inlineStr">
+        <is>
+          <t>https://apccas2025.org/</t>
+        </is>
+      </c>
+      <c r="H42" s="2" t="inlineStr"/>
+      <c r="I42" s="2" t="inlineStr"/>
+      <c r="J42" s="2" t="inlineStr">
+        <is>
+          <t>https://drive.google.com/file/d/1sfqSWkMIY-LUBdyLmo20JaIeud50POEa/view?usp=drive_link</t>
+        </is>
+      </c>
+      <c r="K42" s="2" t="inlineStr"/>
+      <c r="L42" s="2" t="inlineStr">
+        <is>
+          <t>@inproceedings{han2025foscu,
+  title={Foscu: Feasibility of Synthetic Mri Generation Via Duo-Diffusion Models for Enhancement of 3D U-Nets in Hepatic Segmentation},
+  author={Han, Youngung and Kim, Kyeonghun and Ju, Seoyoung and Jean, Yeonju and Cha, Minkyung and Park, Seohyoung and Jung, Hyeonseok and Kim, Nam-Joon and Jeong, Woo Kyoung and Liao, Ken Ying-Kai and others},
+  booktitle={2025 IEEE Asia Pacific Conference on Circuits and Systems (APCCAS)},
+  pages={1–––––––––––––––––––––––––––––––5},
+  year={2025},
+  organization={IEEE}
+}</t>
+        </is>
+      </c>
+      <c r="M42" s="2" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="N42" s="2" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="O42" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="P42" s="2" t="inlineStr">
+        <is>
+          <t>Conference</t>
+        </is>
+      </c>
+      <c r="Q42" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="R42" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="S42" s="2" t="n">
+        <v>360</v>
+      </c>
+      <c r="T42" s="2" t="inlineStr"/>
+      <c r="U42" s="2" t="inlineStr"/>
+      <c r="V42" s="2" t="inlineStr"/>
+      <c r="W42" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="X42" s="2" t="inlineStr">
+        <is>
+          <t>IMSI WEB_Publications</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="2" t="inlineStr">
+        <is>
+          <t>PUB_019</t>
+        </is>
+      </c>
+      <c r="B43" s="2" t="n">
+        <v>2025</v>
+      </c>
+      <c r="C43" s="2" t="inlineStr">
+        <is>
+          <t>Boundary Guidance for Efficient 3D CT Vision–Language Reasoning</t>
+        </is>
+      </c>
+      <c r="D43" s="2" t="inlineStr">
+        <is>
+          <t>ELAMI Workshop at MICCAI 2025</t>
+        </is>
+      </c>
+      <c r="E43" s="2" t="inlineStr">
+        <is>
+          <t>Soo Yong Kim*, Kyeonghun Kim*, Taejin Kim, Yoonkyoung Chun, Hyungjun Kim, Dayoon Lee, Jeongmin Shin, Pa Hong†, Nam-Joon Kim†</t>
+        </is>
+      </c>
+      <c r="F43" s="2" t="inlineStr">
+        <is>
+          <t>https://drive.google.com/file/d/13YIO9V-VDYWp17jj_XIqw6yQtfTMPc5n/view?usp=sharing</t>
+        </is>
+      </c>
+      <c r="G43" s="2" t="inlineStr">
+        <is>
+          <t>https://hula-ai.github.io/LLM-MI-MICCAI-2025/</t>
+        </is>
+      </c>
+      <c r="H43" s="2" t="inlineStr">
+        <is>
+          <t>3D computed tomography (CT) volumes present unique challenges for multimodal reasoning because vision-language models (VLMs) must align long spatial-temporal contexts with radiological text while remaining memory-efficient. We introduce a novel slice-wise visual-instruction prompting scheme that enhances model performance by overlaying colored outlines around relevant anatomy in each 2D slice within the 3D volume...</t>
+        </is>
+      </c>
+      <c r="I43" s="2" t="inlineStr"/>
+      <c r="J43" s="2" t="inlineStr">
+        <is>
+          <t>https://openreview.net/forum?id=RTLvdpF8nu</t>
+        </is>
+      </c>
+      <c r="K43" s="2" t="inlineStr"/>
+      <c r="L43" s="2" t="inlineStr"/>
+      <c r="M43" s="2" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="N43" s="2" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="O43" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="P43" s="2" t="inlineStr">
+        <is>
+          <t>Conference</t>
+        </is>
+      </c>
+      <c r="Q43" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="R43" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="S43" s="2" t="n">
+        <v>370</v>
+      </c>
+      <c r="T43" s="2" t="inlineStr"/>
+      <c r="U43" s="2" t="inlineStr"/>
+      <c r="V43" s="2" t="inlineStr"/>
+      <c r="W43" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="X43" s="2" t="inlineStr">
+        <is>
+          <t>IMSI WEB_Publications</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="2" t="inlineStr">
+        <is>
+          <t>PUB_018</t>
+        </is>
+      </c>
+      <c r="B44" s="2" t="n">
+        <v>2025</v>
+      </c>
+      <c r="C44" s="2" t="inlineStr">
+        <is>
+          <t>Automated Dental Caries Segmentation in Panoramic Radiographs Using Dual-Stage Deep Learning</t>
+        </is>
+      </c>
+      <c r="D44" s="2" t="inlineStr">
+        <is>
+          <t>Workshop on Machine Learning in Medical Imaging (MLMI), MICCAI 2025</t>
+        </is>
+      </c>
+      <c r="E44" s="2" t="inlineStr">
+        <is>
+          <t>Jihun Kim*, Kyeonghun Kim*, Jong-yeol Lee, Yeongseok Seo, Dohyun Chun†</t>
+        </is>
+      </c>
+      <c r="F44" s="2" t="inlineStr">
+        <is>
+          <t>https://drive.google.com/file/d/1EvcCSE42d-yQFZAHQaIaaYY_8GhOdCCt/view</t>
+        </is>
+      </c>
+      <c r="G44" s="2" t="inlineStr">
+        <is>
+          <t>https://sites.google.com/view/mlmi2025/</t>
+        </is>
+      </c>
+      <c r="H44" s="2" t="inlineStr"/>
+      <c r="I44" s="2" t="inlineStr"/>
+      <c r="J44" s="2" t="inlineStr"/>
+      <c r="K44" s="2" t="inlineStr"/>
+      <c r="L44" s="2" t="inlineStr">
+        <is>
+          <t>@inproceedings{kim2025automated,
+  title={Automated Dental Caries Segmentation in Panoramic Radiographs Using Dual-Stage Deep Learning},
+  author={Kim, Jihun and Kim, Kyeonghun and Lee, Jong-yeol and Seo, Yeongseok and Chun, Dohyun},
+  booktitle={International Workshop on Machine Learning in Medical Imaging},
+  pages={551–––––––––––––––––––––––––––––––561},
+  year={2025},
+  organization={Springer}
+}</t>
+        </is>
+      </c>
+      <c r="M44" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="N44" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="O44" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="P44" s="2" t="inlineStr">
+        <is>
+          <t>Conference</t>
+        </is>
+      </c>
+      <c r="Q44" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="R44" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="S44" s="2" t="n">
+        <v>380</v>
+      </c>
+      <c r="T44" s="2" t="inlineStr"/>
+      <c r="U44" s="2" t="inlineStr"/>
+      <c r="V44" s="2" t="inlineStr"/>
+      <c r="W44" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="X44" s="2" t="inlineStr">
+        <is>
+          <t>IMSI WEB_Publications</t>
+        </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:X1"/>
+  <autoFilter ref="A1:X44"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
feat: drive portfolio profile from content model
</commit_message>
<xml_diff>
--- a/docs/Portfolio_Website_Content_Model.xlsx
+++ b/docs/Portfolio_Website_Content_Model.xlsx
@@ -24,9 +24,9 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'README'!$A$1:$B$8</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Site_Config'!$A$1:$E$8</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Site_Config'!$A$1:$E$9</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Home_Sections'!$A$1:$G$3</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'CV_Content'!$A$1:$Q$32</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'CV_Content'!$A$1:$T$44</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Experience_Education'!$A$1:$L$5</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'DB_People'!$A$1:$H$109</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'WEB_Publications'!$A$1:$T$44</definedName>
@@ -2873,7 +2873,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E8"/>
+  <dimension ref="A1:E9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -3063,32 +3063,59 @@
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
+          <t>content_model_url</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>/docs/Portfolio_Website_Content_Model.xlsx</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>/docs/Portfolio_Website_Content_Model.xlsx</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>url</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>Replace with the private Google Sheet URL after upload.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
           <t>public_email</t>
         </is>
       </c>
-      <c r="B8" s="2" t="inlineStr">
+      <c r="B9" s="2" t="inlineStr">
         <is>
           <t>khkim1729@gmail.com</t>
         </is>
       </c>
-      <c r="C8" s="2" t="inlineStr">
+      <c r="C9" s="2" t="inlineStr">
         <is>
           <t>khkim1729@gmail.com</t>
         </is>
       </c>
-      <c r="D8" s="2" t="inlineStr">
+      <c r="D9" s="2" t="inlineStr">
         <is>
           <t>email</t>
         </is>
       </c>
-      <c r="E8" s="2" t="inlineStr">
+      <c r="E9" s="2" t="inlineStr">
         <is>
           <t>Public contact email; do not add a phone number.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:E8"/>
+  <autoFilter ref="A1:E9"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -3226,7 +3253,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q32"/>
+  <dimension ref="A1:T44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -3246,6 +3273,9 @@
     <col width="18" customWidth="1" min="15" max="15"/>
     <col width="18" customWidth="1" min="16" max="16"/>
     <col width="18" customWidth="1" min="17" max="17"/>
+    <col width="18" customWidth="1" min="18" max="18"/>
+    <col width="18" customWidth="1" min="19" max="19"/>
+    <col width="18" customWidth="1" min="20" max="20"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -3326,10 +3356,25 @@
       </c>
       <c r="P1" s="1" t="inlineStr">
         <is>
+          <t>image_url</t>
+        </is>
+      </c>
+      <c r="Q1" s="1" t="inlineStr">
+        <is>
+          <t>image_alt_en</t>
+        </is>
+      </c>
+      <c r="R1" s="1" t="inlineStr">
+        <is>
+          <t>image_alt_ko</t>
+        </is>
+      </c>
+      <c r="S1" s="1" t="inlineStr">
+        <is>
           <t>display_order</t>
         </is>
       </c>
-      <c r="Q1" s="1" t="inlineStr">
+      <c r="T1" s="1" t="inlineStr">
         <is>
           <t>is_visible</t>
         </is>
@@ -3403,10 +3448,13 @@
       </c>
       <c r="N2" s="2" t="inlineStr"/>
       <c r="O2" s="2" t="inlineStr"/>
-      <c r="P2" s="2" t="n">
+      <c r="P2" s="2" t="inlineStr"/>
+      <c r="Q2" s="2" t="inlineStr"/>
+      <c r="R2" s="2" t="inlineStr"/>
+      <c r="S2" s="2" t="n">
         <v>10</v>
       </c>
-      <c r="Q2" s="2" t="b">
+      <c r="T2" s="2" t="b">
         <v>1</v>
       </c>
     </row>
@@ -3480,10 +3528,13 @@
       </c>
       <c r="N3" s="2" t="inlineStr"/>
       <c r="O3" s="2" t="inlineStr"/>
-      <c r="P3" s="2" t="n">
+      <c r="P3" s="2" t="inlineStr"/>
+      <c r="Q3" s="2" t="inlineStr"/>
+      <c r="R3" s="2" t="inlineStr"/>
+      <c r="S3" s="2" t="n">
         <v>20</v>
       </c>
-      <c r="Q3" s="2" t="b">
+      <c r="T3" s="2" t="b">
         <v>1</v>
       </c>
     </row>
@@ -3545,20 +3596,18 @@
       </c>
       <c r="L4" s="2" t="inlineStr">
         <is>
-          <t>Advisor: Prof. Nam-Joon Kim (SNU) and Prof. Wonjae Lee, Radiologist (Samsung Medical Center)
-Lead the SUDAL Medical Imaging Team, organizing weekly journal clubs and mentoring junior researchers
-Built the official IMSI Lab website from the ground up
-Conduct research on conditional abdominal MRI synthesis using segmentation-guided ControlNet pipelines
-Collaborate with Samsung Medical Center radiologists and NVIDIA researchers on medical AI projects</t>
+          <t>Lead the SUDAL Medical Imaging Team and mentor junior researchers across multimodal medical AI projects
+First author of 3D-LLDM, developed with Stanford, NVIDIA, and Samsung Medical Center collaborators and presented orally at IEEE ISBI 2026
+Built and maintain the official IMSI Lab website
+Led an IMSI Lab Silicon Valley programme with office tours and research meetings at Google, NVIDIA San Jose, Salesforce, Uber, Microsoft, and Stanford</t>
         </is>
       </c>
       <c r="M4" s="2" t="inlineStr">
         <is>
-          <t>지도교수: 김남준 교수(서울대학교), 이원재 교수·영상의학과 전문의(삼성서울병원)
-SUDAL 의료영상팀을 이끌며 주간 저널클럽 운영 및 주니어 연구자 멘토링
-IMSI Lab 공식 홈페이지를 처음부터 구축
-분할 정보 기반 ControlNet 파이프라인을 활용한 조건부 복부 MRI 합성 연구
-삼성서울병원 영상의학과 및 NVIDIA 연구진과 의료 AI 프로젝트 협업</t>
+          <t>SUDAL 의료영상팀을 이끌며 멀티모달 의료 AI 프로젝트의 주니어 연구자를 멘토링
+Stanford·NVIDIA·삼성서울병원 연구진과 공동 수행한 3D-LLDM의 제1저자로 IEEE ISBI 2026 구두 발표
+IMSI Lab 공식 홈페이지 구축 및 운영
+IMSI Lab 실리콘밸리 프로그램을 이끌며 Google, NVIDIA San Jose, Salesforce, Uber, Microsoft 및 Stanford 오피스 투어·연구 미팅 진행</t>
         </is>
       </c>
       <c r="N4" s="2" t="inlineStr">
@@ -3567,10 +3616,13 @@
         </is>
       </c>
       <c r="O4" s="2" t="inlineStr"/>
-      <c r="P4" s="2" t="n">
+      <c r="P4" s="2" t="inlineStr"/>
+      <c r="Q4" s="2" t="inlineStr"/>
+      <c r="R4" s="2" t="inlineStr"/>
+      <c r="S4" s="2" t="n">
         <v>100</v>
       </c>
-      <c r="Q4" s="2" t="b">
+      <c r="T4" s="2" t="b">
         <v>1</v>
       </c>
     </row>
@@ -3650,10 +3702,13 @@
         </is>
       </c>
       <c r="O5" s="2" t="inlineStr"/>
-      <c r="P5" s="2" t="n">
+      <c r="P5" s="2" t="inlineStr"/>
+      <c r="Q5" s="2" t="inlineStr"/>
+      <c r="R5" s="2" t="inlineStr"/>
+      <c r="S5" s="2" t="n">
         <v>200</v>
       </c>
-      <c r="Q5" s="2" t="b">
+      <c r="T5" s="2" t="b">
         <v>1</v>
       </c>
     </row>
@@ -3733,10 +3788,13 @@
         </is>
       </c>
       <c r="O6" s="2" t="inlineStr"/>
-      <c r="P6" s="2" t="n">
+      <c r="P6" s="2" t="inlineStr"/>
+      <c r="Q6" s="2" t="inlineStr"/>
+      <c r="R6" s="2" t="inlineStr"/>
+      <c r="S6" s="2" t="n">
         <v>210</v>
       </c>
-      <c r="Q6" s="2" t="b">
+      <c r="T6" s="2" t="b">
         <v>1</v>
       </c>
     </row>
@@ -3814,10 +3872,13 @@
         </is>
       </c>
       <c r="O7" s="2" t="inlineStr"/>
-      <c r="P7" s="2" t="n">
+      <c r="P7" s="2" t="inlineStr"/>
+      <c r="Q7" s="2" t="inlineStr"/>
+      <c r="R7" s="2" t="inlineStr"/>
+      <c r="S7" s="2" t="n">
         <v>220</v>
       </c>
-      <c r="Q7" s="2" t="b">
+      <c r="T7" s="2" t="b">
         <v>1</v>
       </c>
     </row>
@@ -3895,10 +3956,13 @@
         </is>
       </c>
       <c r="O8" s="2" t="inlineStr"/>
-      <c r="P8" s="2" t="n">
+      <c r="P8" s="2" t="inlineStr"/>
+      <c r="Q8" s="2" t="inlineStr"/>
+      <c r="R8" s="2" t="inlineStr"/>
+      <c r="S8" s="2" t="n">
         <v>230</v>
       </c>
-      <c r="Q8" s="2" t="b">
+      <c r="T8" s="2" t="b">
         <v>1</v>
       </c>
     </row>
@@ -3976,10 +4040,13 @@
         </is>
       </c>
       <c r="O9" s="2" t="inlineStr"/>
-      <c r="P9" s="2" t="n">
+      <c r="P9" s="2" t="inlineStr"/>
+      <c r="Q9" s="2" t="inlineStr"/>
+      <c r="R9" s="2" t="inlineStr"/>
+      <c r="S9" s="2" t="n">
         <v>240</v>
       </c>
-      <c r="Q9" s="2" t="b">
+      <c r="T9" s="2" t="b">
         <v>1</v>
       </c>
     </row>
@@ -4057,10 +4124,13 @@
         </is>
       </c>
       <c r="O10" s="2" t="inlineStr"/>
-      <c r="P10" s="2" t="n">
+      <c r="P10" s="2" t="inlineStr"/>
+      <c r="Q10" s="2" t="inlineStr"/>
+      <c r="R10" s="2" t="inlineStr"/>
+      <c r="S10" s="2" t="n">
         <v>250</v>
       </c>
-      <c r="Q10" s="2" t="b">
+      <c r="T10" s="2" t="b">
         <v>1</v>
       </c>
     </row>
@@ -4136,10 +4206,13 @@
         </is>
       </c>
       <c r="O11" s="2" t="inlineStr"/>
-      <c r="P11" s="2" t="n">
+      <c r="P11" s="2" t="inlineStr"/>
+      <c r="Q11" s="2" t="inlineStr"/>
+      <c r="R11" s="2" t="inlineStr"/>
+      <c r="S11" s="2" t="n">
         <v>260</v>
       </c>
-      <c r="Q11" s="2" t="b">
+      <c r="T11" s="2" t="b">
         <v>1</v>
       </c>
     </row>
@@ -4217,10 +4290,13 @@
         </is>
       </c>
       <c r="O12" s="2" t="inlineStr"/>
-      <c r="P12" s="2" t="n">
+      <c r="P12" s="2" t="inlineStr"/>
+      <c r="Q12" s="2" t="inlineStr"/>
+      <c r="R12" s="2" t="inlineStr"/>
+      <c r="S12" s="2" t="n">
         <v>270</v>
       </c>
-      <c r="Q12" s="2" t="b">
+      <c r="T12" s="2" t="b">
         <v>1</v>
       </c>
     </row>
@@ -4296,10 +4372,13 @@
         </is>
       </c>
       <c r="O13" s="2" t="inlineStr"/>
-      <c r="P13" s="2" t="n">
+      <c r="P13" s="2" t="inlineStr"/>
+      <c r="Q13" s="2" t="inlineStr"/>
+      <c r="R13" s="2" t="inlineStr"/>
+      <c r="S13" s="2" t="n">
         <v>280</v>
       </c>
-      <c r="Q13" s="2" t="b">
+      <c r="T13" s="2" t="b">
         <v>1</v>
       </c>
     </row>
@@ -4357,10 +4436,13 @@
       </c>
       <c r="N14" s="2" t="inlineStr"/>
       <c r="O14" s="2" t="inlineStr"/>
-      <c r="P14" s="2" t="n">
+      <c r="P14" s="2" t="inlineStr"/>
+      <c r="Q14" s="2" t="inlineStr"/>
+      <c r="R14" s="2" t="inlineStr"/>
+      <c r="S14" s="2" t="n">
         <v>300</v>
       </c>
-      <c r="Q14" s="2" t="b">
+      <c r="T14" s="2" t="b">
         <v>1</v>
       </c>
     </row>
@@ -4418,10 +4500,13 @@
       </c>
       <c r="N15" s="2" t="inlineStr"/>
       <c r="O15" s="2" t="inlineStr"/>
-      <c r="P15" s="2" t="n">
+      <c r="P15" s="2" t="inlineStr"/>
+      <c r="Q15" s="2" t="inlineStr"/>
+      <c r="R15" s="2" t="inlineStr"/>
+      <c r="S15" s="2" t="n">
         <v>310</v>
       </c>
-      <c r="Q15" s="2" t="b">
+      <c r="T15" s="2" t="b">
         <v>1</v>
       </c>
     </row>
@@ -4481,10 +4566,13 @@
       </c>
       <c r="N16" s="2" t="inlineStr"/>
       <c r="O16" s="2" t="inlineStr"/>
-      <c r="P16" s="2" t="n">
+      <c r="P16" s="2" t="inlineStr"/>
+      <c r="Q16" s="2" t="inlineStr"/>
+      <c r="R16" s="2" t="inlineStr"/>
+      <c r="S16" s="2" t="n">
         <v>400</v>
       </c>
-      <c r="Q16" s="2" t="b">
+      <c r="T16" s="2" t="b">
         <v>1</v>
       </c>
     </row>
@@ -4542,10 +4630,13 @@
       </c>
       <c r="N17" s="2" t="inlineStr"/>
       <c r="O17" s="2" t="inlineStr"/>
-      <c r="P17" s="2" t="n">
+      <c r="P17" s="2" t="inlineStr"/>
+      <c r="Q17" s="2" t="inlineStr"/>
+      <c r="R17" s="2" t="inlineStr"/>
+      <c r="S17" s="2" t="n">
         <v>410</v>
       </c>
-      <c r="Q17" s="2" t="b">
+      <c r="T17" s="2" t="b">
         <v>1</v>
       </c>
     </row>
@@ -4603,10 +4694,13 @@
       </c>
       <c r="N18" s="2" t="inlineStr"/>
       <c r="O18" s="2" t="inlineStr"/>
-      <c r="P18" s="2" t="n">
+      <c r="P18" s="2" t="inlineStr"/>
+      <c r="Q18" s="2" t="inlineStr"/>
+      <c r="R18" s="2" t="inlineStr"/>
+      <c r="S18" s="2" t="n">
         <v>420</v>
       </c>
-      <c r="Q18" s="2" t="b">
+      <c r="T18" s="2" t="b">
         <v>1</v>
       </c>
     </row>
@@ -4643,768 +4737,1129 @@
       </c>
       <c r="G19" s="2" t="inlineStr">
         <is>
-          <t>딥러닝을 이용한 초분광 영상 정제 방법</t>
+          <t>딥러닝을 이용한 초분광이미지의 정제방법</t>
         </is>
       </c>
       <c r="H19" s="2" t="inlineStr">
         <is>
-          <t>Patent Application Filed</t>
+          <t>Registered Patent</t>
         </is>
       </c>
       <c r="I19" s="2" t="inlineStr">
         <is>
-          <t>특허 출원</t>
+          <t>등록 특허</t>
         </is>
       </c>
       <c r="J19" s="2" t="inlineStr">
         <is>
-          <t>Dec. 2024</t>
+          <t>Registered</t>
         </is>
       </c>
       <c r="K19" s="2" t="inlineStr">
         <is>
-          <t>2024년 12월</t>
+          <t>등록 완료</t>
         </is>
       </c>
       <c r="L19" s="2" t="inlineStr">
         <is>
-          <t>Inventors: Hyunjae Park, Seonghun Jeong, Kyeonghun Kim, Taehoon Lim, Dongil Kim
-Application No.: 10-2024-0199713 (Korea)
-Applicant: Gnewsoft Co., Ltd.</t>
+          <t>Registration No.: 10-3010471-0000 (Republic of Korea)
+Inventors: Hyunjae Park, Seonghun Jeong, Kyeonghun Kim, Taehoon Lim, Dongil Kim
+Applicant / Assignee: GNEWSOFT Co., Ltd.</t>
         </is>
       </c>
       <c r="M19" s="2" t="inlineStr">
         <is>
-          <t>발명자: 박현재, 정성훈, 김경훈, 임태훈, 김동일
-출원번호: 10-2024-0199713 (대한민국)
-출원인: 주식회사 지뉴스프트</t>
-        </is>
-      </c>
-      <c r="N19" s="2" t="inlineStr"/>
+          <t>특허등록번호: 10-3010471-0000 (대한민국)
+발명자: 박현재, 정성훈, 김경훈, 임태훈, 김동일
+등록권리자: 주식회사 지뉴스프트</t>
+        </is>
+      </c>
+      <c r="N19" s="2" t="inlineStr">
+        <is>
+          <t>https://www.kipris.or.kr/khome/search/searchResult.do</t>
+        </is>
+      </c>
       <c r="O19" s="2" t="inlineStr"/>
-      <c r="P19" s="2" t="n">
+      <c r="P19" s="2" t="inlineStr"/>
+      <c r="Q19" s="2" t="inlineStr"/>
+      <c r="R19" s="2" t="inlineStr"/>
+      <c r="S19" s="2" t="n">
         <v>500</v>
       </c>
-      <c r="Q19" s="2" t="b">
+      <c r="T19" s="2" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>CV_CRE_001</t>
+          <t>CV_HIL_001</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>credentials</t>
+          <t>highlights</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>Certifications &amp; Licenses</t>
+          <t>Research Highlights</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t>자격증 및 면허</t>
+          <t>연구 하이라이트</t>
         </is>
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>credentials</t>
-        </is>
-      </c>
-      <c r="F20" s="2" t="inlineStr"/>
-      <c r="G20" s="2" t="inlineStr"/>
-      <c r="H20" s="2" t="inlineStr"/>
-      <c r="I20" s="2" t="inlineStr"/>
-      <c r="J20" s="2" t="inlineStr"/>
-      <c r="K20" s="2" t="inlineStr"/>
-      <c r="L20" s="2" t="inlineStr"/>
-      <c r="M20" s="2" t="inlineStr"/>
-      <c r="N20" s="2" t="inlineStr"/>
+          <t>entry</t>
+        </is>
+      </c>
+      <c r="F20" s="2" t="inlineStr">
+        <is>
+          <t>Two Papers Accepted to NeurIPS 2026</t>
+        </is>
+      </c>
+      <c r="G20" s="2" t="inlineStr">
+        <is>
+          <t>NeurIPS 2026 논문 2편 채택</t>
+        </is>
+      </c>
+      <c r="H20" s="2" t="inlineStr">
+        <is>
+          <t>Medical AI reliability and dataset auditing</t>
+        </is>
+      </c>
+      <c r="I20" s="2" t="inlineStr">
+        <is>
+          <t>의료 AI 신뢰성 및 데이터셋 감사</t>
+        </is>
+      </c>
+      <c r="J20" s="2" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="K20" s="2" t="inlineStr">
+        <is>
+          <t>2026년</t>
+        </is>
+      </c>
+      <c r="L20" s="2" t="inlineStr">
+        <is>
+          <t>Co-authored two accepted papers led by Eunseob Choi on correlated failure auditing and Capsule Vision 2024 data auditing.
+Research portfolio also includes 2 MICCAI Workshop papers, 3 ISBI oral papers, 1 IEEE MedAI paper, 3 AICAS oral papers, 4 APCCAS papers, 3 GTC posters, 1 AAAI Workshop paper, and 1 AACL-IJCNLP paper.</t>
+        </is>
+      </c>
+      <c r="M20" s="2" t="inlineStr">
+        <is>
+          <t>최은섭 연구원이 주도한 상관 실패 감사 및 Capsule Vision 2024 데이터 감사 연구 2편의 NeurIPS 2026 채택에 공동저자로 참여했습니다.
+MICCAI Workshop 2편, ISBI 구두발표 3편, IEEE MedAI 1편, AICAS 구두발표 3편, APCCAS 4편, GTC 포스터 3편, AAAI Workshop 1편, AACL-IJCNLP 1편에도 참여했습니다.</t>
+        </is>
+      </c>
+      <c r="N20" s="2" t="inlineStr">
+        <is>
+          <t>https://imsilab.github.io/imsi/news/NEWS-005/</t>
+        </is>
+      </c>
       <c r="O20" s="2" t="inlineStr"/>
-      <c r="P20" s="2" t="n">
-        <v>600</v>
-      </c>
-      <c r="Q20" s="2" t="b">
+      <c r="P20" s="2" t="inlineStr"/>
+      <c r="Q20" s="2" t="inlineStr"/>
+      <c r="R20" s="2" t="inlineStr"/>
+      <c r="S20" s="2" t="n">
+        <v>110</v>
+      </c>
+      <c r="T20" s="2" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>CV_SKL_001</t>
+          <t>CV_LEC_001</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>skills</t>
+          <t>lectures</t>
         </is>
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>Technical Skills</t>
+          <t>Lectures &amp; Teaching</t>
         </is>
       </c>
       <c r="D21" s="2" t="inlineStr">
         <is>
-          <t>기술 역량</t>
+          <t>강의 및 교육</t>
         </is>
       </c>
       <c r="E21" s="2" t="inlineStr">
         <is>
-          <t>skill</t>
+          <t>entry</t>
         </is>
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>Programming Languages</t>
+          <t>Foundational Teaching</t>
         </is>
       </c>
       <c r="G21" s="2" t="inlineStr">
         <is>
-          <t>프로그래밍 언어</t>
+          <t>기초·전공 교육</t>
         </is>
       </c>
       <c r="H21" s="2" t="inlineStr">
         <is>
-          <t>Python, Java, SQL, Bash, C#, JavaScript, TypeScript</t>
+          <t>Fluid mechanics, mechanical engineering, English, TOEFL, Python, machine learning, and deep learning</t>
         </is>
       </c>
       <c r="I21" s="2" t="inlineStr">
         <is>
-          <t>Python, Java, SQL, Bash, C#, JavaScript, TypeScript</t>
-        </is>
-      </c>
-      <c r="J21" s="2" t="inlineStr"/>
-      <c r="K21" s="2" t="inlineStr"/>
-      <c r="L21" s="2" t="inlineStr"/>
-      <c r="M21" s="2" t="inlineStr"/>
+          <t>유체역학, 기계공학개론, 기초 영어, TOEFL, Python, 머신러닝 및 딥러닝</t>
+        </is>
+      </c>
+      <c r="J21" s="2" t="inlineStr">
+        <is>
+          <t>2018 – 2026</t>
+        </is>
+      </c>
+      <c r="K21" s="2" t="inlineStr">
+        <is>
+          <t>2018년 – 2026년</t>
+        </is>
+      </c>
+      <c r="L21" s="2" t="inlineStr">
+        <is>
+          <t>Delivered individual and group instruction spanning engineering fundamentals, language learning, programming, and AI.</t>
+        </is>
+      </c>
+      <c r="M21" s="2" t="inlineStr">
+        <is>
+          <t>공학 기초, 어학, 프로그래밍 및 AI 분야의 개인·그룹 교육을 진행했습니다.</t>
+        </is>
+      </c>
       <c r="N21" s="2" t="inlineStr"/>
       <c r="O21" s="2" t="inlineStr"/>
-      <c r="P21" s="2" t="n">
-        <v>700</v>
-      </c>
-      <c r="Q21" s="2" t="b">
+      <c r="P21" s="2" t="inlineStr"/>
+      <c r="Q21" s="2" t="inlineStr"/>
+      <c r="R21" s="2" t="inlineStr"/>
+      <c r="S21" s="2" t="n">
+        <v>510</v>
+      </c>
+      <c r="T21" s="2" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>CV_SKL_002</t>
+          <t>CV_LEC_002</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>skills</t>
+          <t>lectures</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>Technical Skills</t>
+          <t>Lectures &amp; Teaching</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t>기술 역량</t>
+          <t>강의 및 교육</t>
         </is>
       </c>
       <c r="E22" s="2" t="inlineStr">
         <is>
-          <t>skill</t>
+          <t>entry</t>
         </is>
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>AI/ML Frameworks</t>
+          <t>SK Telecom</t>
         </is>
       </c>
       <c r="G22" s="2" t="inlineStr">
         <is>
-          <t>AI/ML 프레임워크</t>
+          <t>SK텔레콤</t>
         </is>
       </c>
       <c r="H22" s="2" t="inlineStr">
         <is>
-          <t>PyTorch, TensorFlow, MONAI, Hugging Face Transformers, scikit-learn</t>
+          <t>Stable Diffusion for working professionals</t>
         </is>
       </c>
       <c r="I22" s="2" t="inlineStr">
         <is>
-          <t>PyTorch, TensorFlow, MONAI, Hugging Face Transformers, scikit-learn</t>
-        </is>
-      </c>
-      <c r="J22" s="2" t="inlineStr"/>
-      <c r="K22" s="2" t="inlineStr"/>
-      <c r="L22" s="2" t="inlineStr"/>
-      <c r="M22" s="2" t="inlineStr"/>
-      <c r="N22" s="2" t="inlineStr"/>
+          <t>재직자 대상 Stable Diffusion 활용 교육</t>
+        </is>
+      </c>
+      <c r="J22" s="2" t="inlineStr">
+        <is>
+          <t>Dec. 2023</t>
+        </is>
+      </c>
+      <c r="K22" s="2" t="inlineStr">
+        <is>
+          <t>2023년 12월</t>
+        </is>
+      </c>
+      <c r="L22" s="2" t="inlineStr">
+        <is>
+          <t>Three-day hands-on programme covering text-to-image and image-to-image workflows for 30+ engineers.</t>
+        </is>
+      </c>
+      <c r="M22" s="2" t="inlineStr">
+        <is>
+          <t>30명 이상의 엔지니어를 대상으로 Text-to-Image 및 Image-to-Image 실습을 포함한 3일 교육을 진행했습니다.</t>
+        </is>
+      </c>
+      <c r="N22" s="2" t="inlineStr">
+        <is>
+          <t>https://www.sktelecom.com/index_en.html</t>
+        </is>
+      </c>
       <c r="O22" s="2" t="inlineStr"/>
-      <c r="P22" s="2" t="n">
-        <v>710</v>
-      </c>
-      <c r="Q22" s="2" t="b">
+      <c r="P22" s="2" t="inlineStr"/>
+      <c r="Q22" s="2" t="inlineStr"/>
+      <c r="R22" s="2" t="inlineStr"/>
+      <c r="S22" s="2" t="n">
+        <v>520</v>
+      </c>
+      <c r="T22" s="2" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>CV_SKL_003</t>
+          <t>CV_LEC_003</t>
         </is>
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>skills</t>
+          <t>lectures</t>
         </is>
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t>Technical Skills</t>
+          <t>Lectures &amp; Teaching</t>
         </is>
       </c>
       <c r="D23" s="2" t="inlineStr">
         <is>
-          <t>기술 역량</t>
+          <t>강의 및 교육</t>
         </is>
       </c>
       <c r="E23" s="2" t="inlineStr">
         <is>
-          <t>skill</t>
+          <t>entry</t>
         </is>
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>LLM &amp; Vision Models</t>
+          <t>OUTTA AI Bootcamp</t>
         </is>
       </c>
       <c r="G23" s="2" t="inlineStr">
         <is>
-          <t>LLM 및 비전 모델</t>
+          <t>서울대학교 OUTTA AI 부트캠프</t>
         </is>
       </c>
       <c r="H23" s="2" t="inlineStr">
         <is>
-          <t>LLaMA, Gemma VLM, LoRA, RAG, Diffusion Models (DDPM, ControlNet)</t>
+          <t>Python and deep learning instructor</t>
         </is>
       </c>
       <c r="I23" s="2" t="inlineStr">
         <is>
-          <t>LLaMA, Gemma VLM, LoRA, RAG, 확산 모델(DDPM, ControlNet)</t>
-        </is>
-      </c>
-      <c r="J23" s="2" t="inlineStr"/>
-      <c r="K23" s="2" t="inlineStr"/>
-      <c r="L23" s="2" t="inlineStr"/>
-      <c r="M23" s="2" t="inlineStr"/>
-      <c r="N23" s="2" t="inlineStr"/>
+          <t>Python·딥러닝 강사</t>
+        </is>
+      </c>
+      <c r="J23" s="2" t="inlineStr">
+        <is>
+          <t>Jun. 2024 – Aug. 2026</t>
+        </is>
+      </c>
+      <c r="K23" s="2" t="inlineStr">
+        <is>
+          <t>2024년 6월 – 2026년 8월</t>
+        </is>
+      </c>
+      <c r="L23" s="2" t="inlineStr">
+        <is>
+          <t>Delivered recurring AI bootcamp instruction to a cumulative audience of 3,000+ learners.</t>
+        </is>
+      </c>
+      <c r="M23" s="2" t="inlineStr">
+        <is>
+          <t>누적 3,000명 이상의 학습자를 대상으로 AI 부트캠프 강의를 진행했습니다.</t>
+        </is>
+      </c>
+      <c r="N23" s="2" t="inlineStr">
+        <is>
+          <t>https://outta.ai/</t>
+        </is>
+      </c>
       <c r="O23" s="2" t="inlineStr"/>
-      <c r="P23" s="2" t="n">
-        <v>720</v>
-      </c>
-      <c r="Q23" s="2" t="b">
+      <c r="P23" s="2" t="inlineStr">
+        <is>
+          <t>/assets/img/portfolio/lectures/outta-ai-bootcamp.jpg</t>
+        </is>
+      </c>
+      <c r="Q23" s="2" t="inlineStr">
+        <is>
+          <t>OUTTA AI Bootcamp lecture portfolio page</t>
+        </is>
+      </c>
+      <c r="R23" s="2" t="inlineStr">
+        <is>
+          <t>OUTTA AI 부트캠프 강의 포트폴리오</t>
+        </is>
+      </c>
+      <c r="S23" s="2" t="n">
+        <v>530</v>
+      </c>
+      <c r="T23" s="2" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>CV_SKL_004</t>
+          <t>CV_LEC_004</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>skills</t>
+          <t>lectures</t>
         </is>
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>Technical Skills</t>
+          <t>Lectures &amp; Teaching</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>기술 역량</t>
+          <t>강의 및 교육</t>
         </is>
       </c>
       <c r="E24" s="2" t="inlineStr">
         <is>
-          <t>skill</t>
+          <t>entry</t>
         </is>
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
-          <t>Backend &amp; Infrastructure</t>
+          <t>HUN Company</t>
         </is>
       </c>
       <c r="G24" s="2" t="inlineStr">
         <is>
-          <t>백엔드 및 인프라</t>
+          <t>일산 HUN Company</t>
         </is>
       </c>
       <c r="H24" s="2" t="inlineStr">
         <is>
-          <t>Django, FastAPI, Node.js, Nginx, Gunicorn, Docker, Kubernetes</t>
+          <t>Practical ChatGPT for planners</t>
         </is>
       </c>
       <c r="I24" s="2" t="inlineStr">
         <is>
-          <t>Django, FastAPI, Node.js, Nginx, Gunicorn, Docker, Kubernetes</t>
-        </is>
-      </c>
-      <c r="J24" s="2" t="inlineStr"/>
-      <c r="K24" s="2" t="inlineStr"/>
-      <c r="L24" s="2" t="inlineStr"/>
-      <c r="M24" s="2" t="inlineStr"/>
+          <t>기획자를 위한 ChatGPT 실전 활용</t>
+        </is>
+      </c>
+      <c r="J24" s="2" t="inlineStr">
+        <is>
+          <t>Apr. 2025</t>
+        </is>
+      </c>
+      <c r="K24" s="2" t="inlineStr">
+        <is>
+          <t>2025년 4월</t>
+        </is>
+      </c>
+      <c r="L24" s="2" t="inlineStr">
+        <is>
+          <t>Practical generative-AI and prompt-engineering training for working professionals.</t>
+        </is>
+      </c>
+      <c r="M24" s="2" t="inlineStr">
+        <is>
+          <t>재직자를 대상으로 생성형 AI와 프롬프트 엔지니어링 실습 교육을 진행했습니다.</t>
+        </is>
+      </c>
       <c r="N24" s="2" t="inlineStr"/>
       <c r="O24" s="2" t="inlineStr"/>
-      <c r="P24" s="2" t="n">
-        <v>730</v>
-      </c>
-      <c r="Q24" s="2" t="b">
+      <c r="P24" s="2" t="inlineStr"/>
+      <c r="Q24" s="2" t="inlineStr"/>
+      <c r="R24" s="2" t="inlineStr"/>
+      <c r="S24" s="2" t="n">
+        <v>540</v>
+      </c>
+      <c r="T24" s="2" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>CV_SKL_005</t>
+          <t>CV_LEC_005</t>
         </is>
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>skills</t>
+          <t>lectures</t>
         </is>
       </c>
       <c r="C25" s="2" t="inlineStr">
         <is>
-          <t>Technical Skills</t>
+          <t>Lectures &amp; Teaching</t>
         </is>
       </c>
       <c r="D25" s="2" t="inlineStr">
         <is>
-          <t>기술 역량</t>
+          <t>강의 및 교육</t>
         </is>
       </c>
       <c r="E25" s="2" t="inlineStr">
         <is>
-          <t>skill</t>
+          <t>entry</t>
         </is>
       </c>
       <c r="F25" s="2" t="inlineStr">
         <is>
-          <t>Specialized Domains</t>
+          <t>KCA / Kyobo Life</t>
         </is>
       </c>
       <c r="G25" s="2" t="inlineStr">
         <is>
-          <t>전문 분야</t>
+          <t>KCA 교보생명</t>
         </is>
       </c>
       <c r="H25" s="2" t="inlineStr">
         <is>
-          <t>Hyperspectral Imaging, Medical Imaging, Spectral Analysis, Anomaly Detection</t>
+          <t>AX insight and prompt engineering</t>
         </is>
       </c>
       <c r="I25" s="2" t="inlineStr">
         <is>
-          <t>초분광 영상, 의료영상, 분광 분석, 이상 탐지</t>
-        </is>
-      </c>
-      <c r="J25" s="2" t="inlineStr"/>
-      <c r="K25" s="2" t="inlineStr"/>
-      <c r="L25" s="2" t="inlineStr"/>
-      <c r="M25" s="2" t="inlineStr"/>
+          <t>AX 인사이트 및 프롬프트 엔지니어링</t>
+        </is>
+      </c>
+      <c r="J25" s="2" t="inlineStr">
+        <is>
+          <t>Apr. 2026</t>
+        </is>
+      </c>
+      <c r="K25" s="2" t="inlineStr">
+        <is>
+          <t>2026년 4월</t>
+        </is>
+      </c>
+      <c r="L25" s="2" t="inlineStr">
+        <is>
+          <t>Introduced ChatGPT, Gemini, prompt engineering, and custom Gems to 37 employees.</t>
+        </is>
+      </c>
+      <c r="M25" s="2" t="inlineStr">
+        <is>
+          <t>재직자 37명에게 ChatGPT, Gemini, 프롬프트 엔지니어링 및 Gems 제작을 교육했습니다.</t>
+        </is>
+      </c>
       <c r="N25" s="2" t="inlineStr"/>
       <c r="O25" s="2" t="inlineStr"/>
-      <c r="P25" s="2" t="n">
-        <v>740</v>
-      </c>
-      <c r="Q25" s="2" t="b">
+      <c r="P25" s="2" t="inlineStr">
+        <is>
+          <t>/assets/img/portfolio/lectures/kca-kyobo-life.jpg</t>
+        </is>
+      </c>
+      <c r="Q25" s="2" t="inlineStr">
+        <is>
+          <t>KCA Kyobo Life AX lecture portfolio page</t>
+        </is>
+      </c>
+      <c r="R25" s="2" t="inlineStr">
+        <is>
+          <t>KCA 교보생명 AX 강의 포트폴리오</t>
+        </is>
+      </c>
+      <c r="S25" s="2" t="n">
+        <v>550</v>
+      </c>
+      <c r="T25" s="2" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>CV_SKL_006</t>
+          <t>CV_LEC_006</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>skills</t>
+          <t>lectures</t>
         </is>
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>Technical Skills</t>
+          <t>Lectures &amp; Teaching</t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr">
         <is>
-          <t>기술 역량</t>
+          <t>강의 및 교육</t>
         </is>
       </c>
       <c r="E26" s="2" t="inlineStr">
         <is>
-          <t>skill</t>
+          <t>entry</t>
         </is>
       </c>
       <c r="F26" s="2" t="inlineStr">
         <is>
-          <t>Tools</t>
+          <t>Busan Metropolitan City</t>
         </is>
       </c>
       <c r="G26" s="2" t="inlineStr">
         <is>
-          <t>도구</t>
+          <t>부산광역시청</t>
         </is>
       </c>
       <c r="H26" s="2" t="inlineStr">
         <is>
-          <t>Git, Linux, VS Code, PyCharm, Docker Compose, Unity</t>
+          <t>Public-data ideation and advanced prompt engineering</t>
         </is>
       </c>
       <c r="I26" s="2" t="inlineStr">
         <is>
-          <t>Git, Linux, VS Code, PyCharm, Docker Compose, Unity</t>
-        </is>
-      </c>
-      <c r="J26" s="2" t="inlineStr"/>
-      <c r="K26" s="2" t="inlineStr"/>
-      <c r="L26" s="2" t="inlineStr"/>
-      <c r="M26" s="2" t="inlineStr"/>
-      <c r="N26" s="2" t="inlineStr"/>
+          <t>공공데이터 활용 아이디어 도출 및 고급 프롬프트 엔지니어링</t>
+        </is>
+      </c>
+      <c r="J26" s="2" t="inlineStr">
+        <is>
+          <t>Jul. 2026</t>
+        </is>
+      </c>
+      <c r="K26" s="2" t="inlineStr">
+        <is>
+          <t>2026년 7월</t>
+        </is>
+      </c>
+      <c r="L26" s="2" t="inlineStr">
+        <is>
+          <t>Workshop for 36 public officials on public-data platforms, ChatGPT, and evidence-based service ideation.</t>
+        </is>
+      </c>
+      <c r="M26" s="2" t="inlineStr">
+        <is>
+          <t>공무원 36명을 대상으로 공공데이터 플랫폼, ChatGPT 및 근거 기반 서비스 기획 교육을 진행했습니다.</t>
+        </is>
+      </c>
+      <c r="N26" s="2" t="inlineStr">
+        <is>
+          <t>https://www.busan.go.kr/eng/index</t>
+        </is>
+      </c>
       <c r="O26" s="2" t="inlineStr"/>
-      <c r="P26" s="2" t="n">
-        <v>750</v>
-      </c>
-      <c r="Q26" s="2" t="b">
+      <c r="P26" s="2" t="inlineStr">
+        <is>
+          <t>/assets/img/portfolio/lectures/busan-city-hall.jpg</t>
+        </is>
+      </c>
+      <c r="Q26" s="2" t="inlineStr">
+        <is>
+          <t>Busan City Hall public-data lecture portfolio page</t>
+        </is>
+      </c>
+      <c r="R26" s="2" t="inlineStr">
+        <is>
+          <t>부산시청 공공데이터 강의 포트폴리오</t>
+        </is>
+      </c>
+      <c r="S26" s="2" t="n">
+        <v>560</v>
+      </c>
+      <c r="T26" s="2" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>CV_CON_001</t>
+          <t>CV_LEC_007</t>
         </is>
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>contact</t>
+          <t>lectures</t>
         </is>
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>Contact Information</t>
+          <t>Lectures &amp; Teaching</t>
         </is>
       </c>
       <c r="D27" s="2" t="inlineStr">
         <is>
-          <t>연락처</t>
+          <t>강의 및 교육</t>
         </is>
       </c>
       <c r="E27" s="2" t="inlineStr">
         <is>
-          <t>link</t>
+          <t>entry</t>
         </is>
       </c>
       <c r="F27" s="2" t="inlineStr">
         <is>
-          <t>Email</t>
+          <t>Kookmin University AX-Startup Bootcamp</t>
         </is>
       </c>
       <c r="G27" s="2" t="inlineStr">
         <is>
-          <t>이메일</t>
-        </is>
-      </c>
-      <c r="H27" s="2" t="inlineStr"/>
-      <c r="I27" s="2" t="inlineStr"/>
-      <c r="J27" s="2" t="inlineStr"/>
-      <c r="K27" s="2" t="inlineStr"/>
-      <c r="L27" s="2" t="inlineStr"/>
-      <c r="M27" s="2" t="inlineStr"/>
+          <t>국민대학교 AX-Startup 부트캠프</t>
+        </is>
+      </c>
+      <c r="H27" s="2" t="inlineStr">
+        <is>
+          <t>AI literacy and prompt engineering</t>
+        </is>
+      </c>
+      <c r="I27" s="2" t="inlineStr">
+        <is>
+          <t>AI 리터러시 및 프롬프트 엔지니어링</t>
+        </is>
+      </c>
+      <c r="J27" s="2" t="inlineStr">
+        <is>
+          <t>2026.08.29 and 2026.09.01</t>
+        </is>
+      </c>
+      <c r="K27" s="2" t="inlineStr">
+        <is>
+          <t>2026년 8월 29일·9월 1일</t>
+        </is>
+      </c>
+      <c r="L27" s="2" t="inlineStr">
+        <is>
+          <t>Two-session bootcamp on AI literacy, generative AI, and practical prompt engineering for university participants.</t>
+        </is>
+      </c>
+      <c r="M27" s="2" t="inlineStr">
+        <is>
+          <t>대학생 참가자를 대상으로 AI 리터러시, 생성형 AI 및 실전 프롬프트 엔지니어링 2회차 강의를 진행했습니다.</t>
+        </is>
+      </c>
       <c r="N27" s="2" t="inlineStr">
         <is>
-          <t>mailto:khkim1729@gmail.com</t>
-        </is>
-      </c>
-      <c r="O27" s="2" t="inlineStr">
-        <is>
-          <t>📧</t>
-        </is>
-      </c>
-      <c r="P27" s="2" t="n">
-        <v>800</v>
-      </c>
-      <c r="Q27" s="2" t="b">
+          <t>https://english.kookmin.ac.kr/</t>
+        </is>
+      </c>
+      <c r="O27" s="2" t="inlineStr"/>
+      <c r="P27" s="2" t="inlineStr">
+        <is>
+          <t>/assets/img/portfolio/lectures/kookmin-ax-startup.jpg</t>
+        </is>
+      </c>
+      <c r="Q27" s="2" t="inlineStr">
+        <is>
+          <t>Kookmin University AX-Startup Bootcamp portfolio page</t>
+        </is>
+      </c>
+      <c r="R27" s="2" t="inlineStr">
+        <is>
+          <t>국민대학교 AX-Startup 부트캠프 포트폴리오</t>
+        </is>
+      </c>
+      <c r="S27" s="2" t="n">
+        <v>570</v>
+      </c>
+      <c r="T27" s="2" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>CV_CON_002</t>
+          <t>CV_VOL_001</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>contact</t>
+          <t>volunteering</t>
         </is>
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>Contact Information</t>
+          <t>Volunteering &amp; Giving</t>
         </is>
       </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
-          <t>연락처</t>
+          <t>봉사 및 나눔</t>
         </is>
       </c>
       <c r="E28" s="2" t="inlineStr">
         <is>
-          <t>link</t>
+          <t>entry</t>
         </is>
       </c>
       <c r="F28" s="2" t="inlineStr">
         <is>
-          <t>GitHub</t>
+          <t>Blood Donation Volunteer</t>
         </is>
       </c>
       <c r="G28" s="2" t="inlineStr">
         <is>
-          <t>GitHub</t>
-        </is>
-      </c>
-      <c r="H28" s="2" t="inlineStr"/>
-      <c r="I28" s="2" t="inlineStr"/>
-      <c r="J28" s="2" t="inlineStr"/>
-      <c r="K28" s="2" t="inlineStr"/>
-      <c r="L28" s="2" t="inlineStr"/>
-      <c r="M28" s="2" t="inlineStr"/>
+          <t>헌혈 봉사</t>
+        </is>
+      </c>
+      <c r="H28" s="2" t="inlineStr">
+        <is>
+          <t>Korean Red Cross Blood Services</t>
+        </is>
+      </c>
+      <c r="I28" s="2" t="inlineStr">
+        <is>
+          <t>대한적십자사 혈액관리본부</t>
+        </is>
+      </c>
+      <c r="J28" s="2" t="inlineStr">
+        <is>
+          <t>2018 – Present</t>
+        </is>
+      </c>
+      <c r="K28" s="2" t="inlineStr">
+        <is>
+          <t>2018년 – 현재</t>
+        </is>
+      </c>
+      <c r="L28" s="2" t="inlineStr">
+        <is>
+          <t>Completed more than 50 blood donations and continues to donate regularly.</t>
+        </is>
+      </c>
+      <c r="M28" s="2" t="inlineStr">
+        <is>
+          <t>헌혈 50회를 넘겨 현재까지 정기적으로 참여하고 있습니다.</t>
+        </is>
+      </c>
       <c r="N28" s="2" t="inlineStr">
         <is>
-          <t>https://github.com/khkim1729</t>
-        </is>
-      </c>
-      <c r="O28" s="2" t="inlineStr">
-        <is>
-          <t>💻</t>
-        </is>
-      </c>
-      <c r="P28" s="2" t="n">
-        <v>810</v>
-      </c>
-      <c r="Q28" s="2" t="b">
+          <t>https://www.redcross.or.kr/main/main.do</t>
+        </is>
+      </c>
+      <c r="O28" s="2" t="inlineStr"/>
+      <c r="P28" s="2" t="inlineStr"/>
+      <c r="Q28" s="2" t="inlineStr"/>
+      <c r="R28" s="2" t="inlineStr"/>
+      <c r="S28" s="2" t="n">
+        <v>610</v>
+      </c>
+      <c r="T28" s="2" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>CV_CON_003</t>
+          <t>CV_VOL_002</t>
         </is>
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>contact</t>
+          <t>volunteering</t>
         </is>
       </c>
       <c r="C29" s="2" t="inlineStr">
         <is>
-          <t>Contact Information</t>
+          <t>Volunteering &amp; Giving</t>
         </is>
       </c>
       <c r="D29" s="2" t="inlineStr">
         <is>
-          <t>연락처</t>
+          <t>봉사 및 나눔</t>
         </is>
       </c>
       <c r="E29" s="2" t="inlineStr">
         <is>
-          <t>link</t>
+          <t>entry</t>
         </is>
       </c>
       <c r="F29" s="2" t="inlineStr">
         <is>
-          <t>LinkedIn</t>
+          <t>Silver Blood Donation Merit Award</t>
         </is>
       </c>
       <c r="G29" s="2" t="inlineStr">
         <is>
-          <t>LinkedIn</t>
-        </is>
-      </c>
-      <c r="H29" s="2" t="inlineStr"/>
-      <c r="I29" s="2" t="inlineStr"/>
-      <c r="J29" s="2" t="inlineStr"/>
-      <c r="K29" s="2" t="inlineStr"/>
-      <c r="L29" s="2" t="inlineStr"/>
-      <c r="M29" s="2" t="inlineStr"/>
+          <t>헌혈유공장 은장</t>
+        </is>
+      </c>
+      <c r="H29" s="2" t="inlineStr">
+        <is>
+          <t>Korean Red Cross</t>
+        </is>
+      </c>
+      <c r="I29" s="2" t="inlineStr">
+        <is>
+          <t>대한적십자사</t>
+        </is>
+      </c>
+      <c r="J29" s="2" t="inlineStr">
+        <is>
+          <t>2020.10.08</t>
+        </is>
+      </c>
+      <c r="K29" s="2" t="inlineStr">
+        <is>
+          <t>2020.10.08</t>
+        </is>
+      </c>
+      <c r="L29" s="2" t="inlineStr">
+        <is>
+          <t>Recognition for sustained voluntary blood donation.</t>
+        </is>
+      </c>
+      <c r="M29" s="2" t="inlineStr">
+        <is>
+          <t>지속적인 헌혈 참여 공로를 인정받았습니다.</t>
+        </is>
+      </c>
       <c r="N29" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/in/kyeonghun-kim-50705525b/</t>
-        </is>
-      </c>
-      <c r="O29" s="2" t="inlineStr">
-        <is>
-          <t>🔗</t>
-        </is>
-      </c>
-      <c r="P29" s="2" t="n">
-        <v>820</v>
-      </c>
-      <c r="Q29" s="2" t="b">
+          <t>https://www.redcross.or.kr/main/main.do</t>
+        </is>
+      </c>
+      <c r="O29" s="2" t="inlineStr"/>
+      <c r="P29" s="2" t="inlineStr">
+        <is>
+          <t>/assets/img/portfolio/volunteering/blood-silver.jpg</t>
+        </is>
+      </c>
+      <c r="Q29" s="2" t="inlineStr">
+        <is>
+          <t>Korean Red Cross silver blood donation merit award</t>
+        </is>
+      </c>
+      <c r="R29" s="2" t="inlineStr">
+        <is>
+          <t>대한적십자사 헌혈유공장 은장</t>
+        </is>
+      </c>
+      <c r="S29" s="2" t="n">
+        <v>620</v>
+      </c>
+      <c r="T29" s="2" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>CV_CON_004</t>
+          <t>CV_VOL_003</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>contact</t>
+          <t>volunteering</t>
         </is>
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>Contact Information</t>
+          <t>Volunteering &amp; Giving</t>
         </is>
       </c>
       <c r="D30" s="2" t="inlineStr">
         <is>
-          <t>연락처</t>
+          <t>봉사 및 나눔</t>
         </is>
       </c>
       <c r="E30" s="2" t="inlineStr">
         <is>
-          <t>link</t>
+          <t>entry</t>
         </is>
       </c>
       <c r="F30" s="2" t="inlineStr">
         <is>
-          <t>Google Scholar</t>
+          <t>Gold Blood Donation Merit Award</t>
         </is>
       </c>
       <c r="G30" s="2" t="inlineStr">
         <is>
-          <t>Google Scholar</t>
-        </is>
-      </c>
-      <c r="H30" s="2" t="inlineStr"/>
-      <c r="I30" s="2" t="inlineStr"/>
-      <c r="J30" s="2" t="inlineStr"/>
-      <c r="K30" s="2" t="inlineStr"/>
-      <c r="L30" s="2" t="inlineStr"/>
-      <c r="M30" s="2" t="inlineStr"/>
+          <t>헌혈유공장 금장</t>
+        </is>
+      </c>
+      <c r="H30" s="2" t="inlineStr">
+        <is>
+          <t>Korean Red Cross</t>
+        </is>
+      </c>
+      <c r="I30" s="2" t="inlineStr">
+        <is>
+          <t>대한적십자사</t>
+        </is>
+      </c>
+      <c r="J30" s="2" t="inlineStr">
+        <is>
+          <t>2021.08.21</t>
+        </is>
+      </c>
+      <c r="K30" s="2" t="inlineStr">
+        <is>
+          <t>2021.08.21</t>
+        </is>
+      </c>
+      <c r="L30" s="2" t="inlineStr">
+        <is>
+          <t>Recognition for sustained voluntary blood donation.</t>
+        </is>
+      </c>
+      <c r="M30" s="2" t="inlineStr">
+        <is>
+          <t>지속적인 헌혈 참여 공로를 인정받았습니다.</t>
+        </is>
+      </c>
       <c r="N30" s="2" t="inlineStr">
         <is>
-          <t>https://scholar.google.com/citations?user=N3LVcyEAAAAJ&amp;hl=ko</t>
-        </is>
-      </c>
-      <c r="O30" s="2" t="inlineStr">
-        <is>
-          <t>🎓</t>
-        </is>
-      </c>
-      <c r="P30" s="2" t="n">
-        <v>830</v>
-      </c>
-      <c r="Q30" s="2" t="b">
+          <t>https://www.redcross.or.kr/main/main.do</t>
+        </is>
+      </c>
+      <c r="O30" s="2" t="inlineStr"/>
+      <c r="P30" s="2" t="inlineStr">
+        <is>
+          <t>/assets/img/portfolio/volunteering/blood-gold.jpg</t>
+        </is>
+      </c>
+      <c r="Q30" s="2" t="inlineStr">
+        <is>
+          <t>Korean Red Cross gold blood donation merit award</t>
+        </is>
+      </c>
+      <c r="R30" s="2" t="inlineStr">
+        <is>
+          <t>대한적십자사 헌혈유공장 금장</t>
+        </is>
+      </c>
+      <c r="S30" s="2" t="n">
+        <v>630</v>
+      </c>
+      <c r="T30" s="2" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>CV_CON_005</t>
+          <t>CV_VOL_004</t>
         </is>
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>contact</t>
+          <t>volunteering</t>
         </is>
       </c>
       <c r="C31" s="2" t="inlineStr">
         <is>
-          <t>Contact Information</t>
+          <t>Volunteering &amp; Giving</t>
         </is>
       </c>
       <c r="D31" s="2" t="inlineStr">
         <is>
-          <t>연락처</t>
+          <t>봉사 및 나눔</t>
         </is>
       </c>
       <c r="E31" s="2" t="inlineStr">
         <is>
-          <t>link</t>
+          <t>entry</t>
         </is>
       </c>
       <c r="F31" s="2" t="inlineStr">
         <is>
-          <t>Blog</t>
+          <t>Recurring Donor</t>
         </is>
       </c>
       <c r="G31" s="2" t="inlineStr">
         <is>
-          <t>블로그</t>
-        </is>
-      </c>
-      <c r="H31" s="2" t="inlineStr"/>
-      <c r="I31" s="2" t="inlineStr"/>
-      <c r="J31" s="2" t="inlineStr"/>
-      <c r="K31" s="2" t="inlineStr"/>
-      <c r="L31" s="2" t="inlineStr"/>
-      <c r="M31" s="2" t="inlineStr"/>
+          <t>정기 후원</t>
+        </is>
+      </c>
+      <c r="H31" s="2" t="inlineStr">
+        <is>
+          <t>NAVER Happy Bean · NAVER Corp</t>
+        </is>
+      </c>
+      <c r="I31" s="2" t="inlineStr">
+        <is>
+          <t>네이버 해피빈 · NAVER Corp</t>
+        </is>
+      </c>
+      <c r="J31" s="2" t="inlineStr">
+        <is>
+          <t>2015 – Present</t>
+        </is>
+      </c>
+      <c r="K31" s="2" t="inlineStr">
+        <is>
+          <t>2015년 – 현재</t>
+        </is>
+      </c>
+      <c r="L31" s="2" t="inlineStr">
+        <is>
+          <t>Sustained small, recurring contributions—beginning with Happy Bean rewards earned through blogging and growing into regular direct donations—to support vulnerable communities.</t>
+        </is>
+      </c>
+      <c r="M31" s="2" t="inlineStr">
+        <is>
+          <t>블로그 활동으로 얻은 해피빈 기부에서 시작해 정기 직접 후원으로 이어가며 취약계층을 꾸준히 지원하고 있습니다.</t>
+        </is>
+      </c>
       <c r="N31" s="2" t="inlineStr">
         <is>
-          <t>https://blog.naver.com/kgh9080</t>
-        </is>
-      </c>
-      <c r="O31" s="2" t="inlineStr">
-        <is>
-          <t>📝</t>
-        </is>
-      </c>
-      <c r="P31" s="2" t="n">
-        <v>840</v>
-      </c>
-      <c r="Q31" s="2" t="b">
+          <t>https://www.navercorp.com/en/main</t>
+        </is>
+      </c>
+      <c r="O31" s="2" t="inlineStr"/>
+      <c r="P31" s="2" t="inlineStr"/>
+      <c r="Q31" s="2" t="inlineStr"/>
+      <c r="R31" s="2" t="inlineStr"/>
+      <c r="S31" s="2" t="n">
+        <v>640</v>
+      </c>
+      <c r="T31" s="2" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>CV_NOTE_001</t>
+          <t>CV_CRE_001</t>
         </is>
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>note</t>
+          <t>credentials</t>
         </is>
       </c>
       <c r="C32" s="2" t="inlineStr">
         <is>
-          <t>Profile</t>
+          <t>Certifications &amp; Licenses</t>
         </is>
       </c>
       <c r="D32" s="2" t="inlineStr">
         <is>
-          <t>소개</t>
+          <t>자격증 및 면허</t>
         </is>
       </c>
       <c r="E32" s="2" t="inlineStr">
         <is>
-          <t>note</t>
+          <t>credentials</t>
         </is>
       </c>
       <c r="F32" s="2" t="inlineStr"/>
@@ -5413,27 +5868,758 @@
       <c r="I32" s="2" t="inlineStr"/>
       <c r="J32" s="2" t="inlineStr"/>
       <c r="K32" s="2" t="inlineStr"/>
-      <c r="L32" s="2" t="inlineStr">
-        <is>
-          <t>My work connects foundations in computer science with advanced AI research, focusing on medical imaging and practical systems that can benefit society. I aim to bridge academic research and real-world clinical solutions.</t>
-        </is>
-      </c>
-      <c r="M32" s="2" t="inlineStr">
-        <is>
-          <t>컴퓨터과학의 기반 위에서 첨단 AI 연구를 수행하며, 의료영상과 사회에 기여할 수 있는 실용적 시스템에 집중하고 있습니다. 학술 연구와 실제 임상 솔루션 사이의 간극을 연결하는 것을 목표로 합니다.</t>
-        </is>
-      </c>
+      <c r="L32" s="2" t="inlineStr"/>
+      <c r="M32" s="2" t="inlineStr"/>
       <c r="N32" s="2" t="inlineStr"/>
       <c r="O32" s="2" t="inlineStr"/>
-      <c r="P32" s="2" t="n">
-        <v>900</v>
-      </c>
-      <c r="Q32" s="2" t="b">
+      <c r="P32" s="2" t="inlineStr"/>
+      <c r="Q32" s="2" t="inlineStr"/>
+      <c r="R32" s="2" t="inlineStr"/>
+      <c r="S32" s="2" t="n">
+        <v>600</v>
+      </c>
+      <c r="T32" s="2" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="2" t="inlineStr">
+        <is>
+          <t>CV_SKL_001</t>
+        </is>
+      </c>
+      <c r="B33" s="2" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C33" s="2" t="inlineStr">
+        <is>
+          <t>Technical Skills</t>
+        </is>
+      </c>
+      <c r="D33" s="2" t="inlineStr">
+        <is>
+          <t>기술 역량</t>
+        </is>
+      </c>
+      <c r="E33" s="2" t="inlineStr">
+        <is>
+          <t>skill</t>
+        </is>
+      </c>
+      <c r="F33" s="2" t="inlineStr">
+        <is>
+          <t>Programming Languages</t>
+        </is>
+      </c>
+      <c r="G33" s="2" t="inlineStr">
+        <is>
+          <t>프로그래밍 언어</t>
+        </is>
+      </c>
+      <c r="H33" s="2" t="inlineStr">
+        <is>
+          <t>Python, Java, SQL, Bash, C#, JavaScript, TypeScript</t>
+        </is>
+      </c>
+      <c r="I33" s="2" t="inlineStr">
+        <is>
+          <t>Python, Java, SQL, Bash, C#, JavaScript, TypeScript</t>
+        </is>
+      </c>
+      <c r="J33" s="2" t="inlineStr"/>
+      <c r="K33" s="2" t="inlineStr"/>
+      <c r="L33" s="2" t="inlineStr"/>
+      <c r="M33" s="2" t="inlineStr"/>
+      <c r="N33" s="2" t="inlineStr"/>
+      <c r="O33" s="2" t="inlineStr"/>
+      <c r="P33" s="2" t="inlineStr"/>
+      <c r="Q33" s="2" t="inlineStr"/>
+      <c r="R33" s="2" t="inlineStr"/>
+      <c r="S33" s="2" t="n">
+        <v>700</v>
+      </c>
+      <c r="T33" s="2" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="2" t="inlineStr">
+        <is>
+          <t>CV_SKL_002</t>
+        </is>
+      </c>
+      <c r="B34" s="2" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C34" s="2" t="inlineStr">
+        <is>
+          <t>Technical Skills</t>
+        </is>
+      </c>
+      <c r="D34" s="2" t="inlineStr">
+        <is>
+          <t>기술 역량</t>
+        </is>
+      </c>
+      <c r="E34" s="2" t="inlineStr">
+        <is>
+          <t>skill</t>
+        </is>
+      </c>
+      <c r="F34" s="2" t="inlineStr">
+        <is>
+          <t>AI/ML Frameworks</t>
+        </is>
+      </c>
+      <c r="G34" s="2" t="inlineStr">
+        <is>
+          <t>AI/ML 프레임워크</t>
+        </is>
+      </c>
+      <c r="H34" s="2" t="inlineStr">
+        <is>
+          <t>PyTorch, TensorFlow, MONAI, Hugging Face Transformers, scikit-learn</t>
+        </is>
+      </c>
+      <c r="I34" s="2" t="inlineStr">
+        <is>
+          <t>PyTorch, TensorFlow, MONAI, Hugging Face Transformers, scikit-learn</t>
+        </is>
+      </c>
+      <c r="J34" s="2" t="inlineStr"/>
+      <c r="K34" s="2" t="inlineStr"/>
+      <c r="L34" s="2" t="inlineStr"/>
+      <c r="M34" s="2" t="inlineStr"/>
+      <c r="N34" s="2" t="inlineStr"/>
+      <c r="O34" s="2" t="inlineStr"/>
+      <c r="P34" s="2" t="inlineStr"/>
+      <c r="Q34" s="2" t="inlineStr"/>
+      <c r="R34" s="2" t="inlineStr"/>
+      <c r="S34" s="2" t="n">
+        <v>710</v>
+      </c>
+      <c r="T34" s="2" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="2" t="inlineStr">
+        <is>
+          <t>CV_SKL_003</t>
+        </is>
+      </c>
+      <c r="B35" s="2" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C35" s="2" t="inlineStr">
+        <is>
+          <t>Technical Skills</t>
+        </is>
+      </c>
+      <c r="D35" s="2" t="inlineStr">
+        <is>
+          <t>기술 역량</t>
+        </is>
+      </c>
+      <c r="E35" s="2" t="inlineStr">
+        <is>
+          <t>skill</t>
+        </is>
+      </c>
+      <c r="F35" s="2" t="inlineStr">
+        <is>
+          <t>LLM &amp; Vision Models</t>
+        </is>
+      </c>
+      <c r="G35" s="2" t="inlineStr">
+        <is>
+          <t>LLM 및 비전 모델</t>
+        </is>
+      </c>
+      <c r="H35" s="2" t="inlineStr">
+        <is>
+          <t>LLaMA, Gemma VLM, LoRA, RAG, Diffusion Models (DDPM, ControlNet)</t>
+        </is>
+      </c>
+      <c r="I35" s="2" t="inlineStr">
+        <is>
+          <t>LLaMA, Gemma VLM, LoRA, RAG, 확산 모델(DDPM, ControlNet)</t>
+        </is>
+      </c>
+      <c r="J35" s="2" t="inlineStr"/>
+      <c r="K35" s="2" t="inlineStr"/>
+      <c r="L35" s="2" t="inlineStr"/>
+      <c r="M35" s="2" t="inlineStr"/>
+      <c r="N35" s="2" t="inlineStr"/>
+      <c r="O35" s="2" t="inlineStr"/>
+      <c r="P35" s="2" t="inlineStr"/>
+      <c r="Q35" s="2" t="inlineStr"/>
+      <c r="R35" s="2" t="inlineStr"/>
+      <c r="S35" s="2" t="n">
+        <v>720</v>
+      </c>
+      <c r="T35" s="2" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="2" t="inlineStr">
+        <is>
+          <t>CV_SKL_004</t>
+        </is>
+      </c>
+      <c r="B36" s="2" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C36" s="2" t="inlineStr">
+        <is>
+          <t>Technical Skills</t>
+        </is>
+      </c>
+      <c r="D36" s="2" t="inlineStr">
+        <is>
+          <t>기술 역량</t>
+        </is>
+      </c>
+      <c r="E36" s="2" t="inlineStr">
+        <is>
+          <t>skill</t>
+        </is>
+      </c>
+      <c r="F36" s="2" t="inlineStr">
+        <is>
+          <t>Backend &amp; Infrastructure</t>
+        </is>
+      </c>
+      <c r="G36" s="2" t="inlineStr">
+        <is>
+          <t>백엔드 및 인프라</t>
+        </is>
+      </c>
+      <c r="H36" s="2" t="inlineStr">
+        <is>
+          <t>Django, FastAPI, Node.js, Nginx, Gunicorn, Docker, Kubernetes</t>
+        </is>
+      </c>
+      <c r="I36" s="2" t="inlineStr">
+        <is>
+          <t>Django, FastAPI, Node.js, Nginx, Gunicorn, Docker, Kubernetes</t>
+        </is>
+      </c>
+      <c r="J36" s="2" t="inlineStr"/>
+      <c r="K36" s="2" t="inlineStr"/>
+      <c r="L36" s="2" t="inlineStr"/>
+      <c r="M36" s="2" t="inlineStr"/>
+      <c r="N36" s="2" t="inlineStr"/>
+      <c r="O36" s="2" t="inlineStr"/>
+      <c r="P36" s="2" t="inlineStr"/>
+      <c r="Q36" s="2" t="inlineStr"/>
+      <c r="R36" s="2" t="inlineStr"/>
+      <c r="S36" s="2" t="n">
+        <v>730</v>
+      </c>
+      <c r="T36" s="2" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="2" t="inlineStr">
+        <is>
+          <t>CV_SKL_005</t>
+        </is>
+      </c>
+      <c r="B37" s="2" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C37" s="2" t="inlineStr">
+        <is>
+          <t>Technical Skills</t>
+        </is>
+      </c>
+      <c r="D37" s="2" t="inlineStr">
+        <is>
+          <t>기술 역량</t>
+        </is>
+      </c>
+      <c r="E37" s="2" t="inlineStr">
+        <is>
+          <t>skill</t>
+        </is>
+      </c>
+      <c r="F37" s="2" t="inlineStr">
+        <is>
+          <t>Specialized Domains</t>
+        </is>
+      </c>
+      <c r="G37" s="2" t="inlineStr">
+        <is>
+          <t>전문 분야</t>
+        </is>
+      </c>
+      <c r="H37" s="2" t="inlineStr">
+        <is>
+          <t>Hyperspectral Imaging, Medical Imaging, Spectral Analysis, Anomaly Detection</t>
+        </is>
+      </c>
+      <c r="I37" s="2" t="inlineStr">
+        <is>
+          <t>초분광 영상, 의료영상, 분광 분석, 이상 탐지</t>
+        </is>
+      </c>
+      <c r="J37" s="2" t="inlineStr"/>
+      <c r="K37" s="2" t="inlineStr"/>
+      <c r="L37" s="2" t="inlineStr"/>
+      <c r="M37" s="2" t="inlineStr"/>
+      <c r="N37" s="2" t="inlineStr"/>
+      <c r="O37" s="2" t="inlineStr"/>
+      <c r="P37" s="2" t="inlineStr"/>
+      <c r="Q37" s="2" t="inlineStr"/>
+      <c r="R37" s="2" t="inlineStr"/>
+      <c r="S37" s="2" t="n">
+        <v>740</v>
+      </c>
+      <c r="T37" s="2" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="2" t="inlineStr">
+        <is>
+          <t>CV_SKL_006</t>
+        </is>
+      </c>
+      <c r="B38" s="2" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C38" s="2" t="inlineStr">
+        <is>
+          <t>Technical Skills</t>
+        </is>
+      </c>
+      <c r="D38" s="2" t="inlineStr">
+        <is>
+          <t>기술 역량</t>
+        </is>
+      </c>
+      <c r="E38" s="2" t="inlineStr">
+        <is>
+          <t>skill</t>
+        </is>
+      </c>
+      <c r="F38" s="2" t="inlineStr">
+        <is>
+          <t>Tools</t>
+        </is>
+      </c>
+      <c r="G38" s="2" t="inlineStr">
+        <is>
+          <t>도구</t>
+        </is>
+      </c>
+      <c r="H38" s="2" t="inlineStr">
+        <is>
+          <t>Git, Linux, VS Code, PyCharm, Docker Compose, Unity</t>
+        </is>
+      </c>
+      <c r="I38" s="2" t="inlineStr">
+        <is>
+          <t>Git, Linux, VS Code, PyCharm, Docker Compose, Unity</t>
+        </is>
+      </c>
+      <c r="J38" s="2" t="inlineStr"/>
+      <c r="K38" s="2" t="inlineStr"/>
+      <c r="L38" s="2" t="inlineStr"/>
+      <c r="M38" s="2" t="inlineStr"/>
+      <c r="N38" s="2" t="inlineStr"/>
+      <c r="O38" s="2" t="inlineStr"/>
+      <c r="P38" s="2" t="inlineStr"/>
+      <c r="Q38" s="2" t="inlineStr"/>
+      <c r="R38" s="2" t="inlineStr"/>
+      <c r="S38" s="2" t="n">
+        <v>750</v>
+      </c>
+      <c r="T38" s="2" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="2" t="inlineStr">
+        <is>
+          <t>CV_CON_001</t>
+        </is>
+      </c>
+      <c r="B39" s="2" t="inlineStr">
+        <is>
+          <t>contact</t>
+        </is>
+      </c>
+      <c r="C39" s="2" t="inlineStr">
+        <is>
+          <t>Contact Information</t>
+        </is>
+      </c>
+      <c r="D39" s="2" t="inlineStr">
+        <is>
+          <t>연락처</t>
+        </is>
+      </c>
+      <c r="E39" s="2" t="inlineStr">
+        <is>
+          <t>link</t>
+        </is>
+      </c>
+      <c r="F39" s="2" t="inlineStr">
+        <is>
+          <t>Email</t>
+        </is>
+      </c>
+      <c r="G39" s="2" t="inlineStr">
+        <is>
+          <t>이메일</t>
+        </is>
+      </c>
+      <c r="H39" s="2" t="inlineStr"/>
+      <c r="I39" s="2" t="inlineStr"/>
+      <c r="J39" s="2" t="inlineStr"/>
+      <c r="K39" s="2" t="inlineStr"/>
+      <c r="L39" s="2" t="inlineStr"/>
+      <c r="M39" s="2" t="inlineStr"/>
+      <c r="N39" s="2" t="inlineStr">
+        <is>
+          <t>mailto:khkim1729@gmail.com</t>
+        </is>
+      </c>
+      <c r="O39" s="2" t="inlineStr">
+        <is>
+          <t>📧</t>
+        </is>
+      </c>
+      <c r="P39" s="2" t="inlineStr"/>
+      <c r="Q39" s="2" t="inlineStr"/>
+      <c r="R39" s="2" t="inlineStr"/>
+      <c r="S39" s="2" t="n">
+        <v>800</v>
+      </c>
+      <c r="T39" s="2" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="2" t="inlineStr">
+        <is>
+          <t>CV_CON_002</t>
+        </is>
+      </c>
+      <c r="B40" s="2" t="inlineStr">
+        <is>
+          <t>contact</t>
+        </is>
+      </c>
+      <c r="C40" s="2" t="inlineStr">
+        <is>
+          <t>Contact Information</t>
+        </is>
+      </c>
+      <c r="D40" s="2" t="inlineStr">
+        <is>
+          <t>연락처</t>
+        </is>
+      </c>
+      <c r="E40" s="2" t="inlineStr">
+        <is>
+          <t>link</t>
+        </is>
+      </c>
+      <c r="F40" s="2" t="inlineStr">
+        <is>
+          <t>GitHub</t>
+        </is>
+      </c>
+      <c r="G40" s="2" t="inlineStr">
+        <is>
+          <t>GitHub</t>
+        </is>
+      </c>
+      <c r="H40" s="2" t="inlineStr"/>
+      <c r="I40" s="2" t="inlineStr"/>
+      <c r="J40" s="2" t="inlineStr"/>
+      <c r="K40" s="2" t="inlineStr"/>
+      <c r="L40" s="2" t="inlineStr"/>
+      <c r="M40" s="2" t="inlineStr"/>
+      <c r="N40" s="2" t="inlineStr">
+        <is>
+          <t>https://github.com/khkim1729</t>
+        </is>
+      </c>
+      <c r="O40" s="2" t="inlineStr">
+        <is>
+          <t>💻</t>
+        </is>
+      </c>
+      <c r="P40" s="2" t="inlineStr"/>
+      <c r="Q40" s="2" t="inlineStr"/>
+      <c r="R40" s="2" t="inlineStr"/>
+      <c r="S40" s="2" t="n">
+        <v>810</v>
+      </c>
+      <c r="T40" s="2" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="2" t="inlineStr">
+        <is>
+          <t>CV_CON_003</t>
+        </is>
+      </c>
+      <c r="B41" s="2" t="inlineStr">
+        <is>
+          <t>contact</t>
+        </is>
+      </c>
+      <c r="C41" s="2" t="inlineStr">
+        <is>
+          <t>Contact Information</t>
+        </is>
+      </c>
+      <c r="D41" s="2" t="inlineStr">
+        <is>
+          <t>연락처</t>
+        </is>
+      </c>
+      <c r="E41" s="2" t="inlineStr">
+        <is>
+          <t>link</t>
+        </is>
+      </c>
+      <c r="F41" s="2" t="inlineStr">
+        <is>
+          <t>LinkedIn</t>
+        </is>
+      </c>
+      <c r="G41" s="2" t="inlineStr">
+        <is>
+          <t>LinkedIn</t>
+        </is>
+      </c>
+      <c r="H41" s="2" t="inlineStr"/>
+      <c r="I41" s="2" t="inlineStr"/>
+      <c r="J41" s="2" t="inlineStr"/>
+      <c r="K41" s="2" t="inlineStr"/>
+      <c r="L41" s="2" t="inlineStr"/>
+      <c r="M41" s="2" t="inlineStr"/>
+      <c r="N41" s="2" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/kyeonghun-kim-50705525b/</t>
+        </is>
+      </c>
+      <c r="O41" s="2" t="inlineStr">
+        <is>
+          <t>🔗</t>
+        </is>
+      </c>
+      <c r="P41" s="2" t="inlineStr"/>
+      <c r="Q41" s="2" t="inlineStr"/>
+      <c r="R41" s="2" t="inlineStr"/>
+      <c r="S41" s="2" t="n">
+        <v>820</v>
+      </c>
+      <c r="T41" s="2" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="2" t="inlineStr">
+        <is>
+          <t>CV_CON_004</t>
+        </is>
+      </c>
+      <c r="B42" s="2" t="inlineStr">
+        <is>
+          <t>contact</t>
+        </is>
+      </c>
+      <c r="C42" s="2" t="inlineStr">
+        <is>
+          <t>Contact Information</t>
+        </is>
+      </c>
+      <c r="D42" s="2" t="inlineStr">
+        <is>
+          <t>연락처</t>
+        </is>
+      </c>
+      <c r="E42" s="2" t="inlineStr">
+        <is>
+          <t>link</t>
+        </is>
+      </c>
+      <c r="F42" s="2" t="inlineStr">
+        <is>
+          <t>Google Scholar</t>
+        </is>
+      </c>
+      <c r="G42" s="2" t="inlineStr">
+        <is>
+          <t>Google Scholar</t>
+        </is>
+      </c>
+      <c r="H42" s="2" t="inlineStr"/>
+      <c r="I42" s="2" t="inlineStr"/>
+      <c r="J42" s="2" t="inlineStr"/>
+      <c r="K42" s="2" t="inlineStr"/>
+      <c r="L42" s="2" t="inlineStr"/>
+      <c r="M42" s="2" t="inlineStr"/>
+      <c r="N42" s="2" t="inlineStr">
+        <is>
+          <t>https://scholar.google.com/citations?user=N3LVcyEAAAAJ&amp;hl=ko</t>
+        </is>
+      </c>
+      <c r="O42" s="2" t="inlineStr">
+        <is>
+          <t>🎓</t>
+        </is>
+      </c>
+      <c r="P42" s="2" t="inlineStr"/>
+      <c r="Q42" s="2" t="inlineStr"/>
+      <c r="R42" s="2" t="inlineStr"/>
+      <c r="S42" s="2" t="n">
+        <v>830</v>
+      </c>
+      <c r="T42" s="2" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="2" t="inlineStr">
+        <is>
+          <t>CV_CON_005</t>
+        </is>
+      </c>
+      <c r="B43" s="2" t="inlineStr">
+        <is>
+          <t>contact</t>
+        </is>
+      </c>
+      <c r="C43" s="2" t="inlineStr">
+        <is>
+          <t>Contact Information</t>
+        </is>
+      </c>
+      <c r="D43" s="2" t="inlineStr">
+        <is>
+          <t>연락처</t>
+        </is>
+      </c>
+      <c r="E43" s="2" t="inlineStr">
+        <is>
+          <t>link</t>
+        </is>
+      </c>
+      <c r="F43" s="2" t="inlineStr">
+        <is>
+          <t>Blog</t>
+        </is>
+      </c>
+      <c r="G43" s="2" t="inlineStr">
+        <is>
+          <t>블로그</t>
+        </is>
+      </c>
+      <c r="H43" s="2" t="inlineStr"/>
+      <c r="I43" s="2" t="inlineStr"/>
+      <c r="J43" s="2" t="inlineStr"/>
+      <c r="K43" s="2" t="inlineStr"/>
+      <c r="L43" s="2" t="inlineStr"/>
+      <c r="M43" s="2" t="inlineStr"/>
+      <c r="N43" s="2" t="inlineStr">
+        <is>
+          <t>https://blog.naver.com/kgh9080</t>
+        </is>
+      </c>
+      <c r="O43" s="2" t="inlineStr">
+        <is>
+          <t>📝</t>
+        </is>
+      </c>
+      <c r="P43" s="2" t="inlineStr"/>
+      <c r="Q43" s="2" t="inlineStr"/>
+      <c r="R43" s="2" t="inlineStr"/>
+      <c r="S43" s="2" t="n">
+        <v>840</v>
+      </c>
+      <c r="T43" s="2" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="2" t="inlineStr">
+        <is>
+          <t>CV_NOTE_001</t>
+        </is>
+      </c>
+      <c r="B44" s="2" t="inlineStr">
+        <is>
+          <t>note</t>
+        </is>
+      </c>
+      <c r="C44" s="2" t="inlineStr">
+        <is>
+          <t>Profile</t>
+        </is>
+      </c>
+      <c r="D44" s="2" t="inlineStr">
+        <is>
+          <t>소개</t>
+        </is>
+      </c>
+      <c r="E44" s="2" t="inlineStr">
+        <is>
+          <t>note</t>
+        </is>
+      </c>
+      <c r="F44" s="2" t="inlineStr"/>
+      <c r="G44" s="2" t="inlineStr"/>
+      <c r="H44" s="2" t="inlineStr"/>
+      <c r="I44" s="2" t="inlineStr"/>
+      <c r="J44" s="2" t="inlineStr"/>
+      <c r="K44" s="2" t="inlineStr"/>
+      <c r="L44" s="2" t="inlineStr">
+        <is>
+          <t>I am an AI researcher at GNEWSOFT and a Research Assistant at IMSI Lab, Seoul National University. My work spans medical imaging, generative AI, multimodal deep learning, and hyperspectral imaging, with an emphasis on research that can move from reproducible experiments to practical clinical systems.</t>
+        </is>
+      </c>
+      <c r="M44" s="2" t="inlineStr">
+        <is>
+          <t>저는 GNEWSOFT AI 연구원이자 서울대학교 IMSI Lab 연구조교로 활동하고 있습니다. 의료영상, 생성형 AI, 멀티모달 딥러닝 및 초분광 영상을 연구하며 재현 가능한 실험을 실제 임상 시스템으로 연결하는 데 집중합니다.</t>
+        </is>
+      </c>
+      <c r="N44" s="2" t="inlineStr"/>
+      <c r="O44" s="2" t="inlineStr"/>
+      <c r="P44" s="2" t="inlineStr"/>
+      <c r="Q44" s="2" t="inlineStr"/>
+      <c r="R44" s="2" t="inlineStr"/>
+      <c r="S44" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="T44" s="2" t="b">
         <v>1</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:Q32"/>
+  <autoFilter ref="A1:T44"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>